<commit_message>
feat: relocate application to Flash Sector 3
Updated application linker configuration to start at
0x0800C000 (STM32F407 Flash Sector 3) with 464 KB
of available application Flash.

Rebuilt, flashed, and verified successful application execution
from the relocated Flash region.
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D02DE20-9DF5-401B-9DDB-282E7C464325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EDE945E-9E02-4BF3-ADD4-B25E048D2ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project_Info" sheetId="1" r:id="rId1"/>
     <sheet name="SHA256_Testing" sheetId="8" r:id="rId2"/>
-    <sheet name="Defect_Log" sheetId="4" r:id="rId3"/>
-    <sheet name="Test_Summary" sheetId="5" r:id="rId4"/>
+    <sheet name="Memory_Linked_Configuration_Tes" sheetId="9" r:id="rId3"/>
+    <sheet name="Defect_Log" sheetId="4" r:id="rId4"/>
+    <sheet name="Test_Summary" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="97">
   <si>
     <t>Field</t>
   </si>
@@ -538,6 +539,41 @@
       </rPr>
       <t>https://emn178.github.io/online-tools/sha256.html</t>
     </r>
+  </si>
+  <si>
+    <t>Test Description</t>
+  </si>
+  <si>
+    <t>MEM-001</t>
+  </si>
+  <si>
+    <r>
+      <t>Relocate application start to STM32F407 Sector 3 (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x0800C000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) by updating the application linker Flash origin</t>
+    </r>
+  </si>
+  <si>
+    <t>Application builds successfully and executes correctly from the relocated Flash region</t>
+  </si>
+  <si>
+    <t>Application rebuilt, programmed successfully, and executed as expected</t>
   </si>
 </sst>
 </file>
@@ -1227,6 +1263,55 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD55151-40F8-416C-98E3-A78CDE29E48B}">
+  <dimension ref="B2:F3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="3" max="4" width="24.77734375" customWidth="1"/>
+    <col min="5" max="5" width="25.88671875" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6" ht="43.2">
+      <c r="B2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" ht="86.4">
+      <c r="B3" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C5A01BE-886C-4DDC-81AD-947C5C4E69CA}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -1306,7 +1391,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E116B88-DD8B-45A5-9B4A-BCF42512281C}">
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>

</xml_diff>

<commit_message>
feat: automate application image size generation
Added a post-build Python utility to extract application image
boundaries from Main_App.elf and generate app_image_info.h.

Automatically generates:
- Application start address
- Application end address
- Application image size

Verified automatic generation during CubeIDE application build.
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EDE945E-9E02-4BF3-ADD4-B25E048D2ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8562604-128D-4AC7-A802-901767D1F9F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project_Info" sheetId="1" r:id="rId1"/>
     <sheet name="SHA256_Testing" sheetId="8" r:id="rId2"/>
-    <sheet name="Memory_Linked_Configuration_Tes" sheetId="9" r:id="rId3"/>
+    <sheet name="Memory_Linked_Config_Test" sheetId="9" r:id="rId3"/>
     <sheet name="Defect_Log" sheetId="4" r:id="rId4"/>
     <sheet name="Test_Summary" sheetId="5" r:id="rId5"/>
   </sheets>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="140">
   <si>
     <t>Field</t>
   </si>
@@ -541,14 +541,17 @@
     </r>
   </si>
   <si>
-    <t>Test Description</t>
-  </si>
-  <si>
     <t>MEM-001</t>
   </si>
   <si>
-    <r>
-      <t>Relocate application start to STM32F407 Sector 3 (</t>
+    <t>Application Memory Relocation</t>
+  </si>
+  <si>
+    <t>Application shall start from the configured Flash Sector 3 address</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Verify application linker configuration is relocated to </t>
     </r>
     <r>
       <rPr>
@@ -558,22 +561,667 @@
       </rPr>
       <t>0x0800C000</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>) by updating the application linker Flash origin</t>
-    </r>
-  </si>
-  <si>
-    <t>Application builds successfully and executes correctly from the relocated Flash region</t>
-  </si>
-  <si>
-    <t>Application rebuilt, programmed successfully, and executed as expected</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Application linker script configured with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FLASH ORIGIN = 0x0800C000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>LENGTH = 464K</t>
+    </r>
+  </si>
+  <si>
+    <t>Build and flash the application, then execute it on STM32F407</t>
+  </si>
+  <si>
+    <t>Application builds successfully and executes correctly from Sector 3</t>
+  </si>
+  <si>
+    <t>Application rebuilt, flashed successfully, and executed as expected from the relocated Flash region</t>
+  </si>
+  <si>
+    <t>MEM-001_Application_Relocation_Sector3.png</t>
+  </si>
+  <si>
+    <t>Confirms runtime operation after linker relocation</t>
+  </si>
+  <si>
+    <t>MEM-002</t>
+  </si>
+  <si>
+    <t>Application Image Boundary</t>
+  </si>
+  <si>
+    <t>Application image start and end shall be determinable from linker output</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_app_image_start</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_app_image_end</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> are generated correctly in the application </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>.map</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> file</t>
+    </r>
+  </si>
+  <si>
+    <t>Application successfully built with linker-generated image boundary symbols</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inspect </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Main_App.map</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> for </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_app_image_start</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_app_image_end</t>
+    </r>
+  </si>
+  <si>
+    <t>Symbols shall be present with valid addresses</t>
+  </si>
+  <si>
+    <r>
+      <t>_app_image_start = 0x0800C000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_app_image_end = 0x0800DA0C</t>
+    </r>
+  </si>
+  <si>
+    <t>MEM-002_App_Image_Boundaries_MAP.png</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Current image size = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x1A0C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = 6668 bytes</t>
+    </r>
+  </si>
+  <si>
+    <t>MEM-003</t>
+  </si>
+  <si>
+    <t>Linker-generated application boundaries shall be present in the final application ELF</t>
+  </si>
+  <si>
+    <t>Verify symbols are retained in the final ELF used for the firmware build</t>
+  </si>
+  <si>
+    <t>Application ELF generated successfully</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Run </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>arm-none-eabi-nm --defined-only Main_App.elf</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and filter for </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_app_image_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> symbols</t>
+    </r>
+  </si>
+  <si>
+    <t>Both symbols shall be present with the expected addresses</t>
+  </si>
+  <si>
+    <t>MEM-003_App_Image_Boundaries_ELF.png</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Confirms boundaries exist in the actual ELF, not only the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>.map</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> file</t>
+    </r>
+  </si>
+  <si>
+    <t>MEM-004</t>
+  </si>
+  <si>
+    <t>Automated Application Image Size Generation</t>
+  </si>
+  <si>
+    <t>Application image boundaries and size shall be automatically derived from the final application ELF</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Verify that the Python build utility extracts </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_app_image_start</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_app_image_end</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> from </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Main_App.elf</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and generates </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>app_image_info.h</t>
+    </r>
+  </si>
+  <si>
+    <t>Application successfully built and linker-generated image boundary symbols are present in the ELF</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Execute </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>generate_app_image_info.py</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Main_App.elf</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> as input and generate </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>app_image_info.h</t>
+    </r>
+  </si>
+  <si>
+    <t>Script shall extract the linker symbols, calculate the image size, and generate the header with correct values</t>
+  </si>
+  <si>
+    <r>
+      <t>_app_image_start = 0x0800C000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_app_image_end = 0x0800DA0C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, image size = 6668 bytes; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>app_image_info.h</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> generated successfully</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Eliminates manual extraction of application size from the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>.map</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> file</t>
+    </r>
+  </si>
+  <si>
+    <t>MEM-004_Automated_Image_Size_Generation.png
+MEM-004_Automated_Image_Size_Generation_2.png</t>
+  </si>
+  <si>
+    <t>MEM-005</t>
+  </si>
+  <si>
+    <t>Automated Image Boundary Generation</t>
+  </si>
+  <si>
+    <t>Application image information shall be automatically generated from the final application ELF</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Verify CubeIDE automatically executes the image-information generation script after an application build and generates the correct </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>app_image_info.h</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Application linker generates </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_app_image_start</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_app_image_end</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; Python generation script configured as a post-build step</t>
+    </r>
+  </si>
+  <si>
+    <t>Clean-build the Application project and observe the post-build command and generated output</t>
+  </si>
+  <si>
+    <t>Post-build script executes successfully and generates correct application start, end, and image size information</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Script executed automatically during CubeIDE build; Start = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x0800C000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, End = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x0800DA0C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, Size = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>6668 bytes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>app_image_info.h</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> generated successfully</t>
+    </r>
+  </si>
+  <si>
+    <t>MEM-005_Automated_Image_Info_PostBuild.png</t>
+  </si>
+  <si>
+    <t>Establishes the verified Application build-to-image-information pipeline</t>
   </si>
 </sst>
 </file>
@@ -630,7 +1278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -655,6 +1303,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1247,49 +1898,77 @@
       <c r="B9" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="C9:F9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD55151-40F8-416C-98E3-A78CDE29E48B}">
-  <dimension ref="B2:F3"/>
+  <dimension ref="A2:K7"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="3" max="4" width="24.77734375" customWidth="1"/>
-    <col min="5" max="5" width="25.88671875" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" customWidth="1"/>
+    <col min="2" max="2" width="17.77734375" customWidth="1"/>
+    <col min="3" max="3" width="20.6640625" customWidth="1"/>
+    <col min="4" max="4" width="21.44140625" customWidth="1"/>
+    <col min="5" max="5" width="20.44140625" customWidth="1"/>
+    <col min="6" max="6" width="23.77734375" customWidth="1"/>
+    <col min="7" max="7" width="22.109375" customWidth="1"/>
+    <col min="8" max="8" width="22.44140625" customWidth="1"/>
+    <col min="10" max="10" width="23.88671875" customWidth="1"/>
+    <col min="11" max="11" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" ht="43.2">
+    <row r="2" spans="1:11">
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="B2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="72">
+      <c r="A3" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="2:6" ht="86.4">
       <c r="B3" s="2" t="s">
         <v>93</v>
       </c>
@@ -1303,11 +1982,167 @@
         <v>96</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>34</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="72">
+      <c r="A4" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="72">
+      <c r="A5" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="99.6">
+      <c r="A6" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="100.8">
+      <c r="A7" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: establish application image boundary and hash access
Added linker-generated application image start and end symbols,
automated image information generation, and bootloader access to
the application Flash image using the generated image size.

Verified:
- Application start: 0x0800C000
- Application end: 0x0800DA0C
- Application size: 6668 bytes
- Application image accessible from bootloader
- SHA-256 digest generated successfully
- Application vector table configured at 0x0800C000
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8562604-128D-4AC7-A802-901767D1F9F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96278C46-B33C-487F-B278-C921C545EE65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project_Info" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="165">
   <si>
     <t>Field</t>
   </si>
@@ -413,33 +413,16 @@
     <t>SHA-DEF-001</t>
   </si>
   <si>
-    <t xml:space="preserve">Component </t>
-  </si>
-  <si>
     <t>SHA-256 Validation</t>
   </si>
   <si>
-    <t>Incorrect expected SHA-256 reference value was initially identified for the 0-byte input during test-vector preparation.</t>
-  </si>
-  <si>
-    <t>Corrected the reference test vector and re-verified the result.</t>
-  </si>
-  <si>
     <t>Impact</t>
   </si>
   <si>
-    <t>No implementation defect.</t>
-  </si>
-  <si>
     <t>Closed</t>
   </si>
   <si>
     <t>Validation Result</t>
-  </si>
-  <si>
-    <t>Incorrect reference value/typographical error in test-vector preparation.
-Reference value: E3B0C44298FC1C149AFBF4C8996FB92427AE41E4649BAE4F1CA495991B7852B8
-Observed Value:  E3B0C44298FC1C149AFBF4C8996FB92427AE41E4649B934CA495991B7852B855</t>
   </si>
   <si>
     <t>SHA256_test002.png</t>
@@ -1222,6 +1205,746 @@
   </si>
   <si>
     <t>Establishes the verified Application build-to-image-information pipeline</t>
+  </si>
+  <si>
+    <t>Steps to Reproduce</t>
+  </si>
+  <si>
+    <t>Application Vector Table / Bootloader Handover</t>
+  </si>
+  <si>
+    <t>Component</t>
+  </si>
+  <si>
+    <t>MEM-DEF-001</t>
+  </si>
+  <si>
+    <t>Incorrect expected SHA-256 reference value was initially identified for the 0-byte input during SHA-256 test-vector preparation.</t>
+  </si>
+  <si>
+    <t>Calculated SHA-256 digest shall match the standard reference value for an empty input.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Calculated value matched the standard empty-input SHA-256 digest, but the initially entered reference value was incorrect. Reference value initially entered: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>E3B0C44298FC1C149AFBF4C8996FB92427AE41E4649BAE4F1CA495991B7852B8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Correct reference value: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>E3B0C44298FC1C149AFBF4C8996FB92427AE41E4649B934CA495991B7852B855</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Incorrect reference value/typographical error during test-vector preparation. SHA-256 implementation was not defective.</t>
+  </si>
+  <si>
+    <t>Initial test result appeared to indicate an implementation mismatch, causing false failure during validation.</t>
+  </si>
+  <si>
+    <t>Corrected the expected reference test vector and re-ran the test.</t>
+  </si>
+  <si>
+    <t>PASS — Corrected reference value matched the calculated SHA-256 result.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Application entered HardFault after Bootloader → Application handover with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>IACCVIOL = 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>PC = 0x00000000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Application should start from </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x0800C000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>VTOR = 0x0800C000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and no fault.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">HardFault occurred with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>HFSR = 0x40000000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>IACCVIOL = 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>PC = 0x00000000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>VTOR = 0x08008000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>FLASH_BASE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> had previously been changed from </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08000000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08008000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> during earlier bootloader practice work. This caused the application vector-table configuration to use the metadata-sector address.</t>
+    </r>
+  </si>
+  <si>
+    <t>Application handover could fail and cause MCU reset.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Restored </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FLASH_BASE = 0x08000000UL</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and configured application vector-table relocation using </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>USER_VECT_TAB_ADDRESS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>VECT_TAB_OFFSET = 0x0000C000U</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PASS — Application runs normally; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>VTOR = 0x0800C000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>HFSR = 0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CFSR = 0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Build and flash the Bootloader and relocated Application. 
+2. Run the Bootloader and allow it to jump to the Application. 
+3. Inspect </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>HFSR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CFSR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>VTOR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> when the fault occurs.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Execute the SHA-256 test for 0-byte input. 
+2. Compare the calculated digest with the prepared reference value. 
+3. Investigate the mismatch against the standard SHA-256 test vector.</t>
+  </si>
+  <si>
+    <t>MEM-006</t>
+  </si>
+  <si>
+    <t>Application Image Boundary and Flash Access</t>
+  </si>
+  <si>
+    <t>Bootloader shall use the configured application image start address and actual image size to access the application firmware stored in Flash</t>
+  </si>
+  <si>
+    <t>Verify that the bootloader accesses the complete application image using the linker-generated image information</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Application linked at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x0800C000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_app_image_start</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_app_image_end</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> verified in </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>.map</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>.elf</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>APP_IMAGE_SIZE = 6668 bytes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; application executes correctly</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Run the bootloader and use </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>APP_IMAGE_START</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>APP_IMAGE_SIZE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to access the application Flash region and calculate its SHA-256 digest</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Bootloader shall access the intended application Flash region from </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x0800C000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> for </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>6668 bytes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and complete the operation successfully</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Bootloader successfully accessed the application image from </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x0800C000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> for </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>6668 bytes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and generated the SHA-256 digest without fault</t>
+    </r>
+  </si>
+  <si>
+    <t>MEM-006_Application_Flash_Image_Access.png</t>
+  </si>
+  <si>
+    <t>Confirms that the linker-generated application boundaries are correctly used at runtime</t>
   </si>
 </sst>
 </file>
@@ -1278,7 +2001,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1295,20 +2018,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1748,7 +2465,7 @@
         <v>34</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>43</v>
@@ -1783,7 +2500,7 @@
         <v>34</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>47</v>
@@ -1809,16 +2526,16 @@
         <v>63</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>52</v>
@@ -1844,16 +2561,16 @@
         <v>64</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>56</v>
@@ -1876,19 +2593,19 @@
         <v>41</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>60</v>
@@ -1896,14 +2613,14 @@
     </row>
     <row r="9" spans="1:11">
       <c r="B9" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
+        <v>85</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1916,7 +2633,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD55151-40F8-416C-98E3-A78CDE29E48B}">
-  <dimension ref="A2:K7"/>
+  <dimension ref="A2:K8"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="17.77734375" customWidth="1"/>
@@ -1967,177 +2684,212 @@
     </row>
     <row r="3" spans="1:11" ht="72">
       <c r="A3" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J3" s="9" t="s">
-        <v>100</v>
+      <c r="J3" s="6" t="s">
+        <v>95</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="72">
       <c r="A4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="H4" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>109</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J4" s="9" t="s">
-        <v>110</v>
+      <c r="J4" s="6" t="s">
+        <v>105</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="72">
       <c r="A5" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>109</v>
+      <c r="H5" s="6" t="s">
+        <v>104</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J5" s="9" t="s">
-        <v>118</v>
+      <c r="J5" s="6" t="s">
+        <v>113</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="99.6">
       <c r="A6" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="H6" s="6" t="s">
         <v>122</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>127</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J6" s="9" t="s">
-        <v>129</v>
+      <c r="J6" s="6" t="s">
+        <v>124</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="100.8">
       <c r="A7" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>137</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J7" s="9" t="s">
-        <v>138</v>
+      <c r="J7" s="6" t="s">
+        <v>133</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>139</v>
+        <v>134</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="129.6">
+      <c r="A8" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -2148,22 +2900,25 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C5A01BE-886C-4DDC-81AD-947C5C4E69CA}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="12.5546875" style="5" customWidth="1"/>
     <col min="2" max="2" width="10.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.21875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="67.109375" style="5" customWidth="1"/>
-    <col min="6" max="6" width="26.33203125" style="5" customWidth="1"/>
-    <col min="7" max="7" width="23.5546875" style="5" customWidth="1"/>
-    <col min="8" max="8" width="8.88671875" style="5"/>
-    <col min="9" max="9" width="10.109375" style="5" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="5"/>
+    <col min="3" max="3" width="14.88671875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="21" style="5" customWidth="1"/>
+    <col min="5" max="5" width="25.6640625" style="5" customWidth="1"/>
+    <col min="6" max="6" width="17.109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="30.88671875" style="5" customWidth="1"/>
+    <col min="8" max="8" width="25.5546875" style="5" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" style="5" customWidth="1"/>
+    <col min="10" max="10" width="17.6640625" style="5" customWidth="1"/>
+    <col min="11" max="11" width="8.88671875" style="5"/>
+    <col min="12" max="12" width="14.77734375" style="5" customWidth="1"/>
+    <col min="13" max="16384" width="8.88671875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="28.8">
+    <row r="1" spans="1:12" ht="28.8">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -2171,58 +2926,115 @@
         <v>23</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>69</v>
+        <v>137</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I1" s="5" t="s">
-        <v>76</v>
+      <c r="L1" s="1" t="s">
+        <v>72</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="6" customFormat="1" ht="100.8">
-      <c r="A2" s="6" t="s">
+    <row r="2" spans="1:12" ht="168">
+      <c r="A2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="8">
         <v>46276</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="D2" s="6" t="s">
+      <c r="C2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>34</v>
+      <c r="L2" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="158.4">
+      <c r="A3" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B3" s="8">
+        <v>46280</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2253,18 +3065,10 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2"/>
-      <c r="B2" s="2">
-        <v>18</v>
-      </c>
-      <c r="C2" s="2">
-        <v>18</v>
-      </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="4">
-        <v>1</v>
-      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="4"/>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2"/>

</xml_diff>

<commit_message>
feat: store application hash in firmware metadata
Implemented runtime firmware metadata storage in Flash Sector 2.

Metadata includes:
- Magic value
- Application image size
- SHA-256 digest
- Firmware version

Added Flash erase and metadata programming support and verified
metadata readback from Sector 2.

Verified:
- Sector 2 erase successful
- Metadata programmed successfully
- Image size = 6668 bytes
- SHA-256 digest read back byte-for-byte identical
- Firmware version = 1
- Metadata magic = 0xDEADBEEF
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96278C46-B33C-487F-B278-C921C545EE65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{203ADEF5-6CC7-4181-8041-ACEE10FB1152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="185">
   <si>
     <t>Field</t>
   </si>
@@ -1945,6 +1945,276 @@
   </si>
   <si>
     <t>Confirms that the linker-generated application boundaries are correctly used at runtime</t>
+  </si>
+  <si>
+    <t>MEM-007</t>
+  </si>
+  <si>
+    <t>Metadata Flash Sector Erase</t>
+  </si>
+  <si>
+    <t>Bootloader shall erase the dedicated metadata sector before writing new firmware metadata</t>
+  </si>
+  <si>
+    <t>Verify that STM32F407 Flash Sector 2 can be erased at runtime without affecting the application Flash region</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Sector 2 reserved for metadata at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08008000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>flash_storage.c/.h</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> implemented; application located from </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x0800C000</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Execute </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FlashStorage_EraseMetadataSector()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and inspect the contents of Sector 2 using GDB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Sector 2 shall be erased and its contents shall read as </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0xFFFFFFFF</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Sector 2 erase completed successfully; GDB verified the metadata area from </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08008000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> through the metadata region as </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0xFFFFFFFF</t>
+    </r>
+  </si>
+  <si>
+    <t>MEM-007_Metadata_Sector_Erase.png</t>
+  </si>
+  <si>
+    <t>Confirms runtime Flash erase operation before metadata programming; application region remains separate</t>
+  </si>
+  <si>
+    <t>MEM-008</t>
+  </si>
+  <si>
+    <t>Firmware Metadata Programming</t>
+  </si>
+  <si>
+    <t>Bootloader shall store the application image metadata in the dedicated Flash sector</t>
+  </si>
+  <si>
+    <t>Verify that the calculated application image size and SHA-256 digest are correctly programmed into Sector 2 and can be read back from Flash</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Sector 2 erased; application image start = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x0800C000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; image size = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>6668 bytes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; SHA-256 digest successfully calculated</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Create metadata in RAM, erase Sector 2, program the 44-byte metadata structure, then read the metadata back from </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08008000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and compare all fields with the RAM copy</t>
+    </r>
+  </si>
+  <si>
+    <t>Flash-stored metadata shall match the metadata generated by the bootloader</t>
+  </si>
+  <si>
+    <r>
+      <t>magic = 0xDEADBEEF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>image_size = 0x1A0C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>version = 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, and all 32 SHA-256 bytes matched the original RAM digest byte-for-byte</t>
+    </r>
+  </si>
+  <si>
+    <t>MEM-008_Metadata_Programming_Readback.png</t>
+  </si>
+  <si>
+    <t>Confirms persistent storage of firmware metadata in dedicated Sector 2</t>
   </si>
 </sst>
 </file>
@@ -2021,11 +2291,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2615,12 +2885,12 @@
       <c r="B9" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2633,7 +2903,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD55151-40F8-416C-98E3-A78CDE29E48B}">
-  <dimension ref="A2:K8"/>
+  <dimension ref="A2:K10"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="17.77734375" customWidth="1"/>
@@ -2890,6 +3160,76 @@
       </c>
       <c r="K8" s="2" t="s">
         <v>164</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="100.8">
+      <c r="A9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="100.8">
+      <c r="A10" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -2960,7 +3300,7 @@
       <c r="A2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="7">
         <v>46276</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -2994,11 +3334,11 @@
         <v>145</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="158.4">
+    <row r="3" spans="1:12" ht="154.80000000000001">
       <c r="A3" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="7">
         <v>46280</v>
       </c>
       <c r="C3" s="2" t="s">

</xml_diff>

<commit_message>
feat: retrieve firmware metadata on boot
Added boot-time retrieval of stored firmware metadata from
Flash Sector 2 through the Flash storage module.

Verified after MCU reset:
- Metadata magic = 0xDEADBEEF
- Application image size = 6668 bytes
- SHA-256 reference digest retrieved correctly
- Firmware version = 1
- Metadata successfully loaded from Flash into RAM
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{203ADEF5-6CC7-4181-8041-ACEE10FB1152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B743D41-77ED-4F81-BF3B-9E74CA86AB01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="195">
   <si>
     <t>Field</t>
   </si>
@@ -2215,6 +2215,114 @@
   </si>
   <si>
     <t>Confirms persistent storage of firmware metadata in dedicated Sector 2</t>
+  </si>
+  <si>
+    <t>MEM-009</t>
+  </si>
+  <si>
+    <t>Boot-Time Metadata Retrieval</t>
+  </si>
+  <si>
+    <t>Bootloader shall retrieve the stored firmware reference information from the dedicated metadata Flash sector during boot</t>
+  </si>
+  <si>
+    <t>Verify that previously stored metadata can be read from Sector 2 after MCU reset and loaded into RAM</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Valid metadata previously programmed in Sector 2 at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08008000</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Reset the MCU, allow the bootloader to execute </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FlashStorage_ReadMetadata()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, then inspect the retrieved metadata fields using the debugger</t>
+    </r>
+  </si>
+  <si>
+    <t>Bootloader shall retrieve the stored magic, application image size, SHA-256 digest, and firmware version correctly</t>
+  </si>
+  <si>
+    <r>
+      <t>magic = 0xDEADBEEF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>image_size = 0x00001A0C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (6668 bytes), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>version = 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, and the 32-byte SHA-256 digest matched the previously stored reference value</t>
+    </r>
+  </si>
+  <si>
+    <t>MEM-009_Boot_Metadata_Retrieval.png</t>
+  </si>
+  <si>
+    <t>Confirms metadata persists across MCU reset and can be retrieved from Flash into RAM</t>
   </si>
 </sst>
 </file>
@@ -2903,7 +3011,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD55151-40F8-416C-98E3-A78CDE29E48B}">
-  <dimension ref="A2:K10"/>
+  <dimension ref="A2:K11"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="17.77734375" customWidth="1"/>
@@ -3230,6 +3338,41 @@
       </c>
       <c r="K10" s="2" t="s">
         <v>184</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="99.6">
+      <c r="A11" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test(secure-boot): validate successful firmware integrity check
- Recalculated application SHA-256 after MCU reset
- Compared calculated digest with stored reference digest
- Verified matching SHA-256 values and memcmp() == 0
- Confirmed successful jump to application
- Added MEM-010 validation evidence
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B743D41-77ED-4F81-BF3B-9E74CA86AB01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA3A28AE-E86E-467D-B20E-F24448CA7F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="214">
   <si>
     <t>Field</t>
   </si>
@@ -2323,6 +2323,63 @@
   </si>
   <si>
     <t>Confirms metadata persists across MCU reset and can be retrieved from Flash into RAM</t>
+  </si>
+  <si>
+    <t>Confirms that application Flash modification is detected through SHA-256 comparison and prevents execution of a corrupted firmware image</t>
+  </si>
+  <si>
+    <t>After intentional modification of application Flash, the bootloader recalculated the SHA-256 and the calculated digest differed from the stored reference digest; application execution was rejected</t>
+  </si>
+  <si>
+    <t>Calculated SHA-256 shall differ from the stored reference SHA-256 and the bootloader shall reject the modified application</t>
+  </si>
+  <si>
+    <t>Intentionally modify or corrupt application Flash contents, reset the MCU, allow the bootloader to recalculate the application SHA-256, then inspect the calculated digest and stored reference digest using the debugger</t>
+  </si>
+  <si>
+    <t>Valid metadata previously stored in Sector 2 at 0x08008000, including the reference SHA-256 digest</t>
+  </si>
+  <si>
+    <t>Verify that intentional corruption of application Flash results in a SHA-256 mismatch with the stored reference value</t>
+  </si>
+  <si>
+    <t>Bootloader shall detect any modification to the application firmware by recalculating and comparing its SHA-256 digest with the stored reference digest</t>
+  </si>
+  <si>
+    <t>Firmware Integrity Verification</t>
+  </si>
+  <si>
+    <t>MEM-010</t>
+  </si>
+  <si>
+    <t>Confirms successful boot-time integrity verification of an unmodified application image and correct handover to the application</t>
+  </si>
+  <si>
+    <t>MEM-010_Firmware_Integrity_Verification_Success.png</t>
+  </si>
+  <si>
+    <t>After MCU reset, the calculated SHA-256 matched the stored reference SHA-256; memcmp() returned 0 and the bootloader successfully jumped to the application</t>
+  </si>
+  <si>
+    <t>Calculated SHA-256 shall match the stored reference SHA-256 and the bootloader shall accept the application and execute jump_to_application()</t>
+  </si>
+  <si>
+    <t>Reset the MCU, allow the bootloader to calculate the SHA-256 digest of the application Flash, then compare the calculated digest with stored_metadata.sha256 using memcmp()</t>
+  </si>
+  <si>
+    <t>Valid application firmware is programmed in Flash and its reference SHA-256 digest is stored in metadata at 0x08008000</t>
+  </si>
+  <si>
+    <t>Verify that the bootloader successfully validates an unmodified application image after MCU reset</t>
+  </si>
+  <si>
+    <t>Bootloader shall verify the integrity of the application firmware by comparing the calculated SHA-256 digest with the stored reference digest</t>
+  </si>
+  <si>
+    <t>MEM-011</t>
+  </si>
+  <si>
+    <t>MEM-011_Corrupted_Application_Hash.png</t>
   </si>
 </sst>
 </file>
@@ -2379,7 +2436,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2404,6 +2461,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3011,7 +3077,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD55151-40F8-416C-98E3-A78CDE29E48B}">
-  <dimension ref="A2:K11"/>
+  <dimension ref="A2:K13"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="17.77734375" customWidth="1"/>
@@ -3373,6 +3439,76 @@
       </c>
       <c r="K11" s="2" t="s">
         <v>194</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" s="10" customFormat="1" ht="129.6">
+      <c r="A12" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="I12" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="J12" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="K12" s="9" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" s="9" customFormat="1" ht="144">
+      <c r="A13" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="I13" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="J13" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="K13" s="9" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test(secure-boot): validate application hash mismatch
- Modified application behavior to generate a different firmware image
- Rebuilt and programmed the modified application
- Recalculated application SHA-256 after MCU reset
- Verified calculated digest differed from stored reference digest
- Verified modified application was rejected by the bootloader
- Added MEM-011 validation evidence
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA3A28AE-E86E-467D-B20E-F24448CA7F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92FB48AD-634E-4DAB-84CC-F307871E93D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2379,7 +2379,7 @@
     <t>MEM-011</t>
   </si>
   <si>
-    <t>MEM-011_Corrupted_Application_Hash.png</t>
+    <t>MEM-011_Modified_Application_Hash.png</t>
   </si>
 </sst>
 </file>
@@ -2460,9 +2460,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2470,6 +2467,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3059,12 +3059,12 @@
       <c r="B9" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3441,73 +3441,73 @@
         <v>194</v>
       </c>
     </row>
-    <row r="12" spans="1:11" s="10" customFormat="1" ht="129.6">
-      <c r="A12" s="10" t="s">
+    <row r="12" spans="1:11" s="9" customFormat="1" ht="129.6">
+      <c r="A12" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="H12" s="11" t="s">
+      <c r="H12" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="I12" s="9" t="s">
+      <c r="I12" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="J12" s="11" t="s">
+      <c r="J12" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="K12" s="9" t="s">
+      <c r="K12" s="8" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="13" spans="1:11" s="9" customFormat="1" ht="144">
-      <c r="A13" s="9" t="s">
+    <row r="13" spans="1:11" s="8" customFormat="1" ht="144">
+      <c r="A13" s="8" t="s">
         <v>212</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="H13" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="I13" s="9" t="s">
+      <c r="I13" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="J13" s="9" t="s">
+      <c r="J13" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="K13" s="9" t="s">
+      <c r="K13" s="8" t="s">
         <v>195</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(secure-boot): complete firmware integrity verification
- Added application image boundary validation
- Reject application images exceeding the permitted Flash region
- Added firmware metadata magic validation
- Verified successful integrity verification for a valid image
- Verified rejection of a modified application image
- Verified rejection of an invalid application image size
- Added validation evidence for firmware integrity and metadata checks
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92FB48AD-634E-4DAB-84CC-F307871E93D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94EC0F9F-6B87-46F1-9B0B-90085FB6E644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="234">
   <si>
     <t>Field</t>
   </si>
@@ -2380,6 +2380,66 @@
   </si>
   <si>
     <t>MEM-011_Modified_Application_Hash.png</t>
+  </si>
+  <si>
+    <t>Confirms that the bootloader rejects an application image exceeding the permitted Flash region before integrity verification and application handover</t>
+  </si>
+  <si>
+    <t>MEM-012_Invalid_Application_Size.png</t>
+  </si>
+  <si>
+    <t>Bootloader shall detect the invalid image size, enter the error path, and prevent SHA-256 calculation and application execution</t>
+  </si>
+  <si>
+    <t>Using GDB, temporarily modify stored_metadata.image_size to 0x74001, which exceeds the permitted APP_REGION_SIZE of 0x74000, then continue bootloader execution</t>
+  </si>
+  <si>
+    <t>Valid metadata is loaded from Sector 2 and APP_REGION_SIZE is configured for the permitted application Flash region</t>
+  </si>
+  <si>
+    <t>Verify that the bootloader detects an oversized application image and prevents further firmware verification and execution</t>
+  </si>
+  <si>
+    <t>Bootloader shall reject an application image whose declared image size exceeds the permitted application Flash region</t>
+  </si>
+  <si>
+    <t>Image Boundary Validation</t>
+  </si>
+  <si>
+    <t>MEM-012</t>
+  </si>
+  <si>
+    <t>Confirms that the bootloader verifies the metadata record before using firmware image information</t>
+  </si>
+  <si>
+    <t>MEM-013_Invalid_Metadata_Magic.png</t>
+  </si>
+  <si>
+    <t>Bootloader shall detect the invalid magic value, report metadata validation failure, and prevent further image verification and application execution</t>
+  </si>
+  <si>
+    <t>Temporarily modify stored_metadata.magic to an invalid value using the debugger, then reset/continue bootloader execution and observe the metadata validation result</t>
+  </si>
+  <si>
+    <t>Valid firmware metadata is stored in Sector 2 with magic = 0xDEADBEEF</t>
+  </si>
+  <si>
+    <t>Bootloader shall validate the firmware metadata identifier before using metadata contents</t>
+  </si>
+  <si>
+    <t>Metadata Validation</t>
+  </si>
+  <si>
+    <t>Invalid magic value was detected by the bootloader; execution entered the metadata validation error path and the application was not executed</t>
+  </si>
+  <si>
+    <t>Verify that the bootloader detects an invalid metadata magic value and rejects the metadata</t>
+  </si>
+  <si>
+    <t>MEM-013</t>
+  </si>
+  <si>
+    <t>GDB confirmed stored_metadata.image_size = 0x74001 and APP_REGION_SIZE = 0x74000; the boundary check evaluated true and execution entered the Invalid Application Image Size error path</t>
   </si>
 </sst>
 </file>
@@ -3077,10 +3137,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD55151-40F8-416C-98E3-A78CDE29E48B}">
-  <dimension ref="A2:K13"/>
+  <dimension ref="A2:K15"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="17.77734375" customWidth="1"/>
+    <col min="2" max="2" width="13.77734375" customWidth="1"/>
     <col min="3" max="3" width="20.6640625" customWidth="1"/>
     <col min="4" max="4" width="21.44140625" customWidth="1"/>
     <col min="5" max="5" width="20.44140625" customWidth="1"/>
@@ -3088,7 +3148,7 @@
     <col min="7" max="7" width="22.109375" customWidth="1"/>
     <col min="8" max="8" width="22.44140625" customWidth="1"/>
     <col min="10" max="10" width="23.88671875" customWidth="1"/>
-    <col min="11" max="11" width="15.6640625" customWidth="1"/>
+    <col min="11" max="11" width="17.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:11">
@@ -3509,6 +3569,76 @@
       </c>
       <c r="K13" s="8" t="s">
         <v>195</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" s="8" customFormat="1" ht="144">
+      <c r="A14" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="I14" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" s="8" customFormat="1" ht="100.8">
+      <c r="A15" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="I15" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: relocate active application to sector 5
- Move application flash origin from Sector 3 to Sector 5
- Update vector table offset to 0x00020000
- Allocate active application region from Sector 5 onward
- Verify application builds, flashes, and runs successfully
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94EC0F9F-6B87-46F1-9B0B-90085FB6E644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{082E0A80-E128-46FC-8CC9-E314BE4E3F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,8 +16,9 @@
     <sheet name="Project_Info" sheetId="1" r:id="rId1"/>
     <sheet name="SHA256_Testing" sheetId="8" r:id="rId2"/>
     <sheet name="Memory_Linked_Config_Test" sheetId="9" r:id="rId3"/>
-    <sheet name="Defect_Log" sheetId="4" r:id="rId4"/>
-    <sheet name="Test_Summary" sheetId="5" r:id="rId5"/>
+    <sheet name="Dual_Image_FOTA_Test" sheetId="10" r:id="rId4"/>
+    <sheet name="Defect_Log" sheetId="4" r:id="rId5"/>
+    <sheet name="Test_Summary" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="244">
   <si>
     <t>Field</t>
   </si>
@@ -2440,6 +2441,214 @@
   </si>
   <si>
     <t>GDB confirmed stored_metadata.image_size = 0x74001 and APP_REGION_SIZE = 0x74000; the boundary check evaluated true and execution entered the Invalid Application Image Size error path</t>
+  </si>
+  <si>
+    <t>DIF-001</t>
+  </si>
+  <si>
+    <t>Active Image Relocation</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Active application shall be located at the Sector 5 start address </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08020000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Verify that the application is correctly relocated from Sector 3 to Sector 5 and executes successfully.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Application linker configured with Flash origin </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08020000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>VECT_TAB_OFFSET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> configured as </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x00020000U</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>.isr_vector</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> starts at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08020000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; application is successfully flashed and executes normally after reset.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>.isr_vector</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> located at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08020000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; application flashed successfully and is running as expected.</t>
+    </r>
+  </si>
+  <si>
+    <t>Active application successfully relocated from Sector 3 to Sector 5.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Build the application.
+2. Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>.isr_vector</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> location in the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>.map</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> file.
+3. Flash the application.
+4. Reset the MCU.
+5. Verify application execution.</t>
+    </r>
+  </si>
+  <si>
+    <t>DIF-001_Active_Image_Relocation.png</t>
   </si>
 </sst>
 </file>
@@ -2496,7 +2705,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2530,6 +2739,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3137,7 +3355,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD55151-40F8-416C-98E3-A78CDE29E48B}">
-  <dimension ref="A2:K15"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="13.77734375" customWidth="1"/>
@@ -3147,497 +3365,498 @@
     <col min="6" max="6" width="23.77734375" customWidth="1"/>
     <col min="7" max="7" width="22.109375" customWidth="1"/>
     <col min="8" max="8" width="22.44140625" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" style="13"/>
     <col min="10" max="10" width="23.88671875" customWidth="1"/>
     <col min="11" max="11" width="17.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11">
-      <c r="A2" s="1" t="s">
+    <row r="1" spans="1:11">
+      <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="72">
+      <c r="A2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I2" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="72">
       <c r="A3" s="2" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="I3" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="I3" s="12" t="s">
         <v>34</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="72">
+    <row r="4" spans="1:11" ht="57.6">
       <c r="A4" s="2" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>98</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="12" t="s">
         <v>34</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="72">
+    <row r="5" spans="1:11" ht="99.6">
       <c r="A5" s="2" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>98</v>
+        <v>116</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="I5" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="I5" s="12" t="s">
         <v>34</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="99.6">
+    <row r="6" spans="1:11" ht="100.8">
       <c r="A6" s="2" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="I6" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="I6" s="12" t="s">
         <v>34</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="100.8">
+    <row r="7" spans="1:11" ht="129.6">
       <c r="A7" s="2" t="s">
-        <v>125</v>
+        <v>155</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>126</v>
+        <v>156</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>128</v>
+        <v>158</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>129</v>
+        <v>159</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>130</v>
+        <v>160</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="I7" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="I7" s="12" t="s">
         <v>34</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>133</v>
+        <v>163</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>134</v>
+        <v>164</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="129.6">
+    <row r="8" spans="1:11" ht="100.8">
       <c r="A8" s="2" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="I8" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="I8" s="12" t="s">
         <v>34</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="100.8">
       <c r="A9" s="2" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="I9" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="I9" s="12" t="s">
         <v>34</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="100.8">
+    <row r="10" spans="1:11" ht="99.6">
       <c r="A10" s="2" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="I10" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="I10" s="12" t="s">
         <v>34</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="99.6">
-      <c r="A11" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="I11" s="2" t="s">
+    <row r="11" spans="1:11" s="9" customFormat="1" ht="115.2">
+      <c r="A11" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="I11" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="J11" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>194</v>
+      <c r="J11" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>204</v>
       </c>
     </row>
-    <row r="12" spans="1:11" s="9" customFormat="1" ht="129.6">
-      <c r="A12" s="9" t="s">
-        <v>203</v>
+    <row r="12" spans="1:11" s="8" customFormat="1" ht="129.6">
+      <c r="A12" s="8" t="s">
+        <v>212</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>202</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>207</v>
-      </c>
-      <c r="H12" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="I12" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>196</v>
+      </c>
+      <c r="I12" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="J12" s="10" t="s">
-        <v>205</v>
+      <c r="J12" s="8" t="s">
+        <v>213</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
     </row>
     <row r="13" spans="1:11" s="8" customFormat="1" ht="144">
       <c r="A13" s="8" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>202</v>
+        <v>221</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>201</v>
+        <v>220</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>200</v>
+        <v>219</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>198</v>
+        <v>217</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>196</v>
-      </c>
-      <c r="I13" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="I13" s="12" t="s">
         <v>34</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="K13" s="8" t="s">
-        <v>195</v>
+        <v>214</v>
       </c>
     </row>
-    <row r="14" spans="1:11" s="8" customFormat="1" ht="144">
+    <row r="14" spans="1:11" s="8" customFormat="1" ht="100.8">
       <c r="A14" s="8" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="I14" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="I14" s="12" t="s">
         <v>34</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
       <c r="K14" s="8" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" s="8" customFormat="1" ht="100.8">
-      <c r="A15" s="8" t="s">
-        <v>232</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>229</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>228</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>231</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>227</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>226</v>
-      </c>
-      <c r="G15" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="H15" s="8" t="s">
-        <v>230</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="J15" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="K15" s="8" t="s">
         <v>223</v>
       </c>
     </row>
@@ -3648,6 +3867,99 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD30C987-18E6-4B70-93B6-FCBA274DBA4D}">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="8.88671875" style="14"/>
+    <col min="2" max="2" width="10.5546875" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="22.77734375" customWidth="1"/>
+    <col min="5" max="5" width="23.44140625" customWidth="1"/>
+    <col min="6" max="6" width="26.33203125" customWidth="1"/>
+    <col min="7" max="7" width="22.6640625" customWidth="1"/>
+    <col min="8" max="8" width="21.109375" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" style="13"/>
+    <col min="10" max="10" width="16.21875" customWidth="1"/>
+    <col min="11" max="11" width="17.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="100.8">
+      <c r="A2" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="I2" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C5A01BE-886C-4DDC-81AD-947C5C4E69CA}">
   <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -3787,7 +4099,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E116B88-DD8B-45A5-9B4A-BCF42512281C}">
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>

</xml_diff>

<commit_message>
feat: add candidate firmware image
- Create separate Candidate_App project
- Configure candidate firmware for Sector 4
- Configure vector table at 0x08010000
- Integrate verified SHA-256 implementation
- Add red LED demonstrator application
- Verify repeatable SHA-256 digest generation
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{082E0A80-E128-46FC-8CC9-E314BE4E3F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D24DE7A0-9C32-4780-B2BE-5E115C38DF64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="264">
   <si>
     <t>Field</t>
   </si>
@@ -2649,6 +2649,297 @@
   </si>
   <si>
     <t>DIF-001_Active_Image_Relocation.png</t>
+  </si>
+  <si>
+    <t>DIF-002</t>
+  </si>
+  <si>
+    <t>Candidate Firmware Image</t>
+  </si>
+  <si>
+    <t>Candidate application shall be configured to execute from the Sector 3–4 region and shall contain the SHA-256 implementation and a demonstrator application.</t>
+  </si>
+  <si>
+    <t>Verify that the candidate firmware is correctly linked, located, and executed from its designated Flash region.</t>
+  </si>
+  <si>
+    <t>Candidate project created; candidate linker configured for Sector 4; SHA-256 implementation included; red LED application implemented.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Candidate </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>.isr_vector</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> starts at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08010000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; VTOR points to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08010000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; candidate firmware executes successfully; red LED toggles; SHA-256 implementation is included.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Candidate project created; red LED is glowing. VTOR currently observed at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08020000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, indicating the vector-table offset still requires correction.</t>
+    </r>
+  </si>
+  <si>
+    <t>Initial validation revealed that the candidate project retained the Active Application's vector-table offset. Correct offset and repeat validation before marking PASS.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Configure candidate linker Flash origin as </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08010000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with length </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>64K</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.
+2. Configure </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>VECT_TAB_OFFSET</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> as </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x00010000U</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.
+3. Build the candidate application.
+4. Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>.isr_vector</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> location in the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>.map</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> file.
+5. Flash candidate firmware.
+6. Verify VTOR points to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08010000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.
+7. Verify red LED toggles.
+8. Confirm SHA-256 implementation is included in the build.</t>
+    </r>
+  </si>
+  <si>
+    <t>Candidate application shall be configured to execute from the Sector 3–4 region and shall contain the SHA-256 implementation and a simple demonstrator application.</t>
+  </si>
+  <si>
+    <t>Verify that the candidate firmware is built and executed from the candidate region, contains the SHA-256 implementation, and can calculate a consistent firmware digest.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Candidate project configured for Sector 4; vector table configured for </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08010000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; SHA-256 module integrated; red LED demonstrator implemented.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Build the Candidate application.2. Flash the Candidate firmware.3. Verify the application executes and red LED toggles.4. Run the SHA-256 calculation.5. Record the calculated digest.6. Repeat the calculation and compare the result.</t>
+  </si>
+  <si>
+    <t>Candidate application executes successfully; red LED toggles; SHA-256 calculation completes; repeated calculations produce the same digest.</t>
+  </si>
+  <si>
+    <t>Candidate application built and executed successfully. Red LED toggled. SHA-256 digest was calculated successfully and the same digest was obtained in two separate checks.</t>
+  </si>
+  <si>
+    <t>Candidate firmware successfully established as a separate firmware image with integrated SHA-256 functionality.</t>
+  </si>
+  <si>
+    <t>DIF-003_Candidate_Firmware_SHA256.png</t>
+  </si>
+  <si>
+    <t>Candidate Firmware Image initial validation</t>
+  </si>
+  <si>
+    <t>DIF-002_Candidate_Firmware_Image_Initial_Validation.png</t>
+  </si>
+  <si>
+    <t>DIF-003</t>
   </si>
 </sst>
 </file>
@@ -2738,9 +3029,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2748,6 +3036,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3337,12 +3628,12 @@
       <c r="B9" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3365,7 +3656,7 @@
     <col min="6" max="6" width="23.77734375" customWidth="1"/>
     <col min="7" max="7" width="22.109375" customWidth="1"/>
     <col min="8" max="8" width="22.44140625" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" style="13"/>
+    <col min="9" max="9" width="8.88671875" style="12"/>
     <col min="10" max="10" width="23.88671875" customWidth="1"/>
     <col min="11" max="11" width="17.33203125" customWidth="1"/>
   </cols>
@@ -3430,7 +3721,7 @@
       <c r="H2" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="11" t="s">
         <v>34</v>
       </c>
       <c r="J2" s="6" t="s">
@@ -3465,7 +3756,7 @@
       <c r="H3" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="11" t="s">
         <v>34</v>
       </c>
       <c r="J3" s="6" t="s">
@@ -3500,7 +3791,7 @@
       <c r="H4" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="11" t="s">
         <v>34</v>
       </c>
       <c r="J4" s="6" t="s">
@@ -3535,7 +3826,7 @@
       <c r="H5" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="I5" s="12" t="s">
+      <c r="I5" s="11" t="s">
         <v>34</v>
       </c>
       <c r="J5" s="6" t="s">
@@ -3570,7 +3861,7 @@
       <c r="H6" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="I6" s="11" t="s">
         <v>34</v>
       </c>
       <c r="J6" s="6" t="s">
@@ -3605,7 +3896,7 @@
       <c r="H7" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="I7" s="12" t="s">
+      <c r="I7" s="11" t="s">
         <v>34</v>
       </c>
       <c r="J7" s="6" t="s">
@@ -3640,7 +3931,7 @@
       <c r="H8" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="I8" s="12" t="s">
+      <c r="I8" s="11" t="s">
         <v>34</v>
       </c>
       <c r="J8" s="6" t="s">
@@ -3675,7 +3966,7 @@
       <c r="H9" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="I9" s="12" t="s">
+      <c r="I9" s="11" t="s">
         <v>34</v>
       </c>
       <c r="J9" s="6" t="s">
@@ -3710,7 +4001,7 @@
       <c r="H10" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="11" t="s">
         <v>34</v>
       </c>
       <c r="J10" s="6" t="s">
@@ -3745,7 +4036,7 @@
       <c r="H11" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="I11" s="12" t="s">
+      <c r="I11" s="11" t="s">
         <v>34</v>
       </c>
       <c r="J11" s="10" t="s">
@@ -3780,7 +4071,7 @@
       <c r="H12" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="I12" s="12" t="s">
+      <c r="I12" s="11" t="s">
         <v>34</v>
       </c>
       <c r="J12" s="8" t="s">
@@ -3815,7 +4106,7 @@
       <c r="H13" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="I13" s="12" t="s">
+      <c r="I13" s="11" t="s">
         <v>34</v>
       </c>
       <c r="J13" s="8" t="s">
@@ -3850,7 +4141,7 @@
       <c r="H14" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="I14" s="12" t="s">
+      <c r="I14" s="11" t="s">
         <v>34</v>
       </c>
       <c r="J14" s="8" t="s">
@@ -3868,18 +4159,18 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD30C987-18E6-4B70-93B6-FCBA274DBA4D}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="14"/>
+    <col min="1" max="1" width="8.88671875" style="13"/>
     <col min="2" max="2" width="10.5546875" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="22.77734375" customWidth="1"/>
     <col min="5" max="5" width="23.44140625" customWidth="1"/>
-    <col min="6" max="6" width="26.33203125" customWidth="1"/>
+    <col min="6" max="6" width="33.44140625" customWidth="1"/>
     <col min="7" max="7" width="22.6640625" customWidth="1"/>
     <col min="8" max="8" width="21.109375" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" style="13"/>
+    <col min="9" max="9" width="8.88671875" style="12"/>
     <col min="10" max="10" width="16.21875" customWidth="1"/>
     <col min="11" max="11" width="17.6640625" customWidth="1"/>
   </cols>
@@ -3919,8 +4210,8 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="100.8">
-      <c r="A2" s="12" t="s">
+    <row r="2" spans="1:11" ht="86.4">
+      <c r="A2" s="11" t="s">
         <v>234</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -3944,7 +4235,7 @@
       <c r="H2" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="11" t="s">
         <v>34</v>
       </c>
       <c r="J2" s="2" t="s">
@@ -3952,10 +4243,81 @@
       </c>
       <c r="K2" s="2" t="s">
         <v>241</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="172.8">
+      <c r="A3" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="158.4">
+      <c r="A4" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>259</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: add candidate firmware metadata
- Define candidate firmware metadata structure
- Add image size, version, SHA-256 digest, and update state fields
- Reserve Sector 3 for candidate metadata
- Add candidate metadata flash storage support
- Store candidate metadata after SHA-256 calculation
- Verify stored metadata using GDB
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D24DE7A0-9C32-4780-B2BE-5E115C38DF64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ED2A145-DA08-4A19-9350-9CBB0284A7DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project_Info" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="274">
   <si>
     <t>Field</t>
   </si>
@@ -2940,6 +2940,240 @@
   </si>
   <si>
     <t>DIF-003</t>
+  </si>
+  <si>
+    <t>DIF-004</t>
+  </si>
+  <si>
+    <t>Candidate Firmware Metadata</t>
+  </si>
+  <si>
+    <t>Candidate metadata shall store image size, version, reference SHA-256 digest, and update state in the designated Candidate Metadata region.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Verify that candidate metadata is correctly formatted and stored in Sector 3 at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x0800C000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Candidate firmware is configured for Sector 4; SHA-256 calculation is working; Candidate Metadata is configured for Sector 3.</t>
+  </si>
+  <si>
+    <t>1. Build and flash the Candidate application.2. Allow the application to calculate the SHA-256 digest and populate metadata.3. Read Sector 3 using GDB.4. Verify magic, image size, version, SHA-256 digest, and update state.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Metadata is stored at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x0800C000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>magic = 0xDEADBEEF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; image size matches the candidate image; version is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; stored SHA-256 matches the calculated digest; update state is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>PENDING_VALIDATION</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">GDB confirmed metadata at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x0800C000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>magic = 0xDEADBEEF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>image_size = 0x28EC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (10,476 bytes), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>version = 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, SHA-256 matches the calculated digest, and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>update_state = 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>PENDING_VALIDATION</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <t>DIF-004_Candidate_Metadata.png</t>
+  </si>
+  <si>
+    <t>Candidate metadata successfully stored and verified in Sector 3. Candidate image remains in Sector 4.</t>
   </si>
 </sst>
 </file>
@@ -4159,7 +4393,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD30C987-18E6-4B70-93B6-FCBA274DBA4D}">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="13"/>
@@ -4313,6 +4547,41 @@
       </c>
       <c r="K4" s="2" t="s">
         <v>259</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="158.4">
+      <c r="A5" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement candidate image SHA validation and active fallback
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ED2A145-DA08-4A19-9350-9CBB0284A7DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63EE6B16-7F6B-4078-9D34-0F86D55CEDC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project_Info" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="303">
   <si>
     <t>Field</t>
   </si>
@@ -3174,6 +3174,343 @@
   </si>
   <si>
     <t>Candidate metadata successfully stored and verified in Sector 3. Candidate image remains in Sector 4.</t>
+  </si>
+  <si>
+    <t>DIF-005</t>
+  </si>
+  <si>
+    <t>STM32CubeIDE / ST-LINK Debug</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Flash programming failed during the debug launch sequence with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Error finishing flash operation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. The debugger session terminated before execution could be halted for fault analysis.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Launch the bootloader debug configuration in STM32CubeIDE.2. Attempt to load </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Secure_Boot.elf</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.3. Observe the Flash programming error and debugger termination.4. Repeat using a previously known-working firmware build.5. Connect to the target using STM32CubeProgrammer over SWD.</t>
+    </r>
+  </si>
+  <si>
+    <t>Firmware should be programmed successfully and the debugger session should start normally.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">CubeIDE reported </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Error finishing flash operation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> for both the current and previously working firmware. STM32CubeProgrammer successfully connected to the MCU over SWD.</t>
+    </r>
+  </si>
+  <si>
+    <t>Debug/programming session issue; the same failure with a known-working build indicates it was not caused by the latest firmware changes. Exact underlying CubeIDE/ST-LINK cause was not isolated.</t>
+  </si>
+  <si>
+    <t>Prevented firmware programming and debugger-based fault analysis during validation.</t>
+  </si>
+  <si>
+    <t>Re-established target connection and successfully verified MCU access using STM32CubeProgrammer.</t>
+  </si>
+  <si>
+    <t>Target connectivity and SWD access successfully verified; firmware validation resumed.</t>
+  </si>
+  <si>
+    <t>Active Image Verification During Normal Boot</t>
+  </si>
+  <si>
+    <t>During normal boot, the bootloader shall read and validate Active Image metadata, calculate the SHA-256 digest over the defined Active Image region, compare it with the stored reference digest, and execute the Active Image only when verification succeeds.</t>
+  </si>
+  <si>
+    <t>Verify that the bootloader successfully validates and executes the Active Image when the stored metadata and SHA-256 digest are valid.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Valid Active Image V0 is stored at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08020000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; valid Active metadata is stored in Sector 2; reference SHA-256 matches the current Active Image.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Reset the MCU. Bootloader reads Active metadata, validates the metadata and image boundaries, calculates the Active Image SHA-256, compares the calculated digest with the stored reference digest, and transfers control to the Active Image. Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>SCB-&gt;VTOR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and PC using GDB after handover.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Active metadata is accepted; calculated SHA-256 matches the stored reference digest; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>JumpToApplication()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> executes successfully; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>SCB-&gt;VTOR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> points to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08020000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; PC lies within the Active Image region.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Active metadata and image boundaries were validated successfully. Calculated Active SHA-256 matched the stored reference digest. GDB confirmed </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>SCB-&gt;VTOR = 0x08020000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>PC = 0x08020AC8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; Active firmware executed successfully.</t>
+    </r>
+  </si>
+  <si>
+    <t>Confirms normal-boot integrity verification and controlled handover to the validated Active Image.</t>
+  </si>
+  <si>
+    <t>DIF-005_Active_Image_Verification_During_Normal_Boot.png</t>
+  </si>
+  <si>
+    <t>DIF-006</t>
+  </si>
+  <si>
+    <t>Candidate Image SHA-256 Verification</t>
+  </si>
+  <si>
+    <t>When a candidate image is present, the bootloader shall independently calculate the candidate image SHA-256 digest and compare it with the reference digest stored in Candidate Metadata.</t>
+  </si>
+  <si>
+    <t>Verify that the SHA-256 digest calculated over the Candidate Image in Flash matches the reference digest stored in Sector 3 and that the Candidate Image is accepted only on a match.</t>
+  </si>
+  <si>
+    <t>Candidate firmware V1 is stored in Sector 4; Candidate Metadata is stored in Sector 3; candidate metadata is valid and contains the reference SHA-256 digest.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Reset the MCU.2. Verify candidate metadata is read and validated.3. Confirm candidate version is newer than Active version.4. Verify Candidate Image start, image size, and calculated end address in GDB.5. Calculate Candidate SHA-256 using the defined image range.6. Inspect </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>candidate_digest</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> using GDB.7. Inspect </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>candidate_metadata.sha256</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> from the metadata structure.8. Compare the 32-byte calculated and stored digests.9. Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>SCB-&gt;VTOR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and PC after successful handover.</t>
+    </r>
+  </si>
+  <si>
+    <t>Candidate image boundaries are valid; calculated SHA-256 matches the reference SHA-256 stored in Candidate Metadata; Candidate Image is accepted and execution is transferred to the Candidate Image.</t>
+  </si>
+  <si>
+    <t>Pending execution of the GDB digest comparison and final handover verification.</t>
+  </si>
+  <si>
+    <t>Verifies the complete Candidate Image integrity-check path and confirms that metadata is not included in the SHA-256 calculation.</t>
+  </si>
+  <si>
+    <t>DIF-006_Candidate_Image_SHA-256_Verification.png</t>
   </si>
 </sst>
 </file>
@@ -3230,7 +3567,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3273,6 +3610,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4393,7 +4733,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD30C987-18E6-4B70-93B6-FCBA274DBA4D}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="13"/>
@@ -4584,6 +4924,76 @@
         <v>273</v>
       </c>
     </row>
+    <row r="6" spans="1:11" ht="244.8">
+      <c r="A6" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="201.6">
+      <c r="A7" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>301</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -4592,7 +5002,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C5A01BE-886C-4DDC-81AD-947C5C4E69CA}">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="12.5546875" style="5" customWidth="1"/>
@@ -4722,6 +5132,41 @@
       </c>
       <c r="L3" s="2" t="s">
         <v>152</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="187.2">
+      <c r="B4" s="15">
+        <v>46283</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Simplify FOTA candidate validation and fallback flow
Removed persistent candidate update-state handling from the FOTA boot flow.

The bootloader now:
- Validates active and candidate metadata
- Checks candidate firmware version
- Verifies candidate SHA-256 before boot
- Falls back to active firmware when candidate validation fails
- Enters fail-safe when active firmware integrity verification fails

Update-state based activation and rollback handling is deferred for future enhancement.
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63EE6B16-7F6B-4078-9D34-0F86D55CEDC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A320F884-4DEF-48E9-97F6-3D4986577E91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,8 +17,9 @@
     <sheet name="SHA256_Testing" sheetId="8" r:id="rId2"/>
     <sheet name="Memory_Linked_Config_Test" sheetId="9" r:id="rId3"/>
     <sheet name="Dual_Image_FOTA_Test" sheetId="10" r:id="rId4"/>
-    <sheet name="Defect_Log" sheetId="4" r:id="rId5"/>
-    <sheet name="Test_Summary" sheetId="5" r:id="rId6"/>
+    <sheet name="FOTA Boot Flow Validation" sheetId="11" r:id="rId5"/>
+    <sheet name="Defect_Log" sheetId="4" r:id="rId6"/>
+    <sheet name="Test_Summary" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="409">
   <si>
     <t>Field</t>
   </si>
@@ -3511,6 +3512,1099 @@
   </si>
   <si>
     <t>DIF-006_Candidate_Image_SHA-256_Verification.png</t>
+  </si>
+  <si>
+    <t>SHAT_Testing</t>
+  </si>
+  <si>
+    <t>Memory_Linked_Config_Test</t>
+  </si>
+  <si>
+    <t>Dual_Image_FOTA_Test</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-001</t>
+  </si>
+  <si>
+    <t>Active Metadata Read</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-002</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-003</t>
+  </si>
+  <si>
+    <t>Active Metadata Validation</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-004</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-005</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-006</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-007</t>
+  </si>
+  <si>
+    <t>Candidate Metadata Validation</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-008</t>
+  </si>
+  <si>
+    <t>Candidate Version Check</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-009</t>
+  </si>
+  <si>
+    <t>Candidate SHA-256 Verification</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-010</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-011</t>
+  </si>
+  <si>
+    <t>Active SHA-256 Verification</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-012</t>
+  </si>
+  <si>
+    <t>FOTA Boot Flow Validation</t>
+  </si>
+  <si>
+    <t>Bootloader shall successfully read active image metadata.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FlashStorage_ReadMetadata()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> returns </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>HAL_OK</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Valid active metadata programmed at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FLASH_ACTIVE_METADATA_ADDRESS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; valid active/candidate firmware available.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Run the normal build. Set GDB breakpoint immediately after active metadata read and inspect </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>status</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>status == HAL_OK</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; execution continues to active metadata validation; no fail-safe is entered.</t>
+    </r>
+  </si>
+  <si>
+    <t>Baseline successful read condition.</t>
+  </si>
+  <si>
+    <t>Bootloader shall enter fail-safe when active metadata read fails.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>status != HAL_OK</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> path.</t>
+    </r>
+  </si>
+  <si>
+    <t>Same baseline configuration.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Set GDB breakpoint after </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FlashStorage_ReadMetadata()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Modify </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>status</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>HAL_ERROR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> in GDB and continue execution.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>status != HAL_OK</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; execution enters </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Bootloader_FailSafe()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>GDB-controlled failure injection.</t>
+  </si>
+  <si>
+    <t>Bootloader shall reject invalid active metadata.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Metadata_Validate()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> failure path.</t>
+    </r>
+  </si>
+  <si>
+    <t>Active metadata can be read successfully but contains an invalid field.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Run with valid read status. Modify an active metadata field to an invalid value and inspect the return value of </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Metadata_Validate()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> in GDB.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Metadata_Validate()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> returns false; execution enters </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Bootloader_FailSafe()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Tests invalid active metadata.</t>
+  </si>
+  <si>
+    <t>Bootloader shall continue when active metadata is valid.</t>
+  </si>
+  <si>
+    <t>Verify successful active metadata validation.</t>
+  </si>
+  <si>
+    <t>Valid active metadata.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">During the baseline run, set GDB breakpoint after </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Metadata_Validate()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and inspect the return value.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Metadata_Validate()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> returns true; execution continues to candidate metadata processing.</t>
+    </r>
+  </si>
+  <si>
+    <t>Baseline successful validation condition.</t>
+  </si>
+  <si>
+    <t>Candidate Metadata Read</t>
+  </si>
+  <si>
+    <t>Bootloader shall continue with active-image fallback when candidate metadata cannot be read.</t>
+  </si>
+  <si>
+    <t>Verify candidate metadata read failure path.</t>
+  </si>
+  <si>
+    <t>Active metadata valid; candidate read operation reached.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Set GDB breakpoint after candidate </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FlashStorage_ReadMetadata()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Modify </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>status</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>HAL_ERROR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and continue.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>status != HAL_OK</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>candidate_metadata_valid</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> becomes false; candidate image is not processed; execution continues to active-image verification.</t>
+    </r>
+  </si>
+  <si>
+    <t>Bootloader shall accept valid candidate metadata for further processing.</t>
+  </si>
+  <si>
+    <t>Verify successful candidate metadata read and validation.</t>
+  </si>
+  <si>
+    <t>Valid active and candidate metadata; candidate version newer than active.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">During the baseline run, inspect </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>status</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>candidate_metadata_valid</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and the result of </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Metadata_Validate()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> in GDB.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Candidate read returns </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>HAL_OK</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>candidate_metadata_valid == true</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; execution enters candidate handling.</t>
+    </r>
+  </si>
+  <si>
+    <t>Baseline successful candidate validation condition.</t>
+  </si>
+  <si>
+    <t>Bootloader shall reject invalid candidate metadata.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Verify </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>!candidate_metadata_valid</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> path.</t>
+    </r>
+  </si>
+  <si>
+    <t>Candidate metadata is readable but contains an invalid field.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Keep candidate read successful. Modify/corrupt candidate metadata and inspect </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Metadata_Validate()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> result in GDB.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Candidate metadata validation returns false; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>candidate_metadata_valid == false</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; candidate processing is skipped and active-image verification continues.</t>
+    </r>
+  </si>
+  <si>
+    <t>Tests invalid candidate metadata.</t>
+  </si>
+  <si>
+    <t>Bootloader shall not process a candidate that is not newer than the active image.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Verify false path of </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Metadata_IsCandidateNewer()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Active and candidate metadata are both valid.</t>
+  </si>
+  <si>
+    <t>Use a candidate image whose version is equal to or lower than the active version. Set GDB breakpoint at the version comparison and inspect the result.</t>
+  </si>
+  <si>
+    <r>
+      <t>Metadata_IsCandidateNewer()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> returns false; candidate SHA-256 calculation is skipped; active-image verification continues.</t>
+    </r>
+  </si>
+  <si>
+    <t>Tests candidate-selection decision independently of SHA validation.</t>
+  </si>
+  <si>
+    <t>Bootloader shall boot a newer candidate only when its SHA-256 matches the stored digest.</t>
+  </si>
+  <si>
+    <t>Verify successful candidate integrity verification and candidate execution.</t>
+  </si>
+  <si>
+    <t>Valid active metadata; valid newer candidate; candidate firmware matches stored SHA-256.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Use the baseline valid configuration. Set GDB breakpoint at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ImageValidation_VerifySHA256()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and inspect the result. Continue execution.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SHA verification returns true; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>JumpToApplication()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is called with candidate image; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Red LED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> indicates candidate image execution.</t>
+    </r>
+  </si>
+  <si>
+    <t>Successful candidate boot path.</t>
+  </si>
+  <si>
+    <t>Bootloader shall reject a candidate when its SHA-256 does not match.</t>
+  </si>
+  <si>
+    <t>Verify candidate SHA mismatch path and fallback to active image.</t>
+  </si>
+  <si>
+    <t>Active image valid; candidate metadata valid and newer. Candidate digest must be made invalid.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Modify candidate firmware or stored candidate digest so verification fails. Inspect </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ImageValidation_VerifySHA256()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> result in GDB and continue.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SHA verification returns false; candidate is rejected; active-image SHA verification executes; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Orange LED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> indicates active image execution.</t>
+    </r>
+  </si>
+  <si>
+    <t>Candidate integrity failure with active fallback.</t>
+  </si>
+  <si>
+    <t>Bootloader shall boot the active image when its SHA-256 matches.</t>
+  </si>
+  <si>
+    <t>Verify successful active-image integrity verification and active execution.</t>
+  </si>
+  <si>
+    <t>Active image valid; candidate unavailable, invalid, or not newer.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Set GDB breakpoint at active </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ImageValidation_VerifySHA256()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and inspect the result. Continue execution.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SHA verification returns true; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>JumpToApplication()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is called for active image; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Orange LED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> indicates active image execution.</t>
+    </r>
+  </si>
+  <si>
+    <t>Successful active fallback/normal boot path.</t>
+  </si>
+  <si>
+    <t>Bootloader shall enter fail-safe when active SHA-256 verification fails.</t>
+  </si>
+  <si>
+    <t>Verify active integrity failure handling.</t>
+  </si>
+  <si>
+    <t>Active metadata valid, but active firmware or stored digest is modified so SHA verification fails. Candidate must not successfully boot.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Modify active firmware/digest and inspect the active </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ImageValidation_VerifySHA256()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> result in GDB. Continue execution.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SHA verification returns false; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Bootloader_FailSafe()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is executed; normal active/candidate application is not started.</t>
+    </r>
+  </si>
+  <si>
+    <t>Final fail-safe path.</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-001_Active_Metadata_Read.png</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-002_Active_Metadata_Read_Error.png</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-004_Active_Metadata_Validation_Pass.png</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-006_Candidate_Metadata_Validation_Pass.png</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-003_Active_Metadata_Validation_Fail.png</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-005_Candidate_Metadata_Read_Error.png</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-007_Candidate_Metadata_Validation_Fail.png</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-008_Candidate_Version_Check.png</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-009_Candidate_SHA256_Pass.png</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-010_Candidate_SHA256_Mismatch.png</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-011_Active_SHA256_Pass.png</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-012_Active_SHA256_Mismatch.png</t>
   </si>
 </sst>
 </file>
@@ -3608,11 +4702,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4202,12 +5296,12 @@
       <c r="B9" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5001,6 +6095,484 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05E5142-AEE3-4F3C-9EE7-B4A55C2203BE}">
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="9.6640625" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" customWidth="1"/>
+    <col min="3" max="3" width="21.33203125" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" customWidth="1"/>
+    <col min="5" max="5" width="21.77734375" customWidth="1"/>
+    <col min="6" max="6" width="24.21875" customWidth="1"/>
+    <col min="7" max="7" width="27.21875" customWidth="1"/>
+    <col min="8" max="8" width="22.6640625" customWidth="1"/>
+    <col min="10" max="10" width="21.33203125" customWidth="1"/>
+    <col min="11" max="11" width="17.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="85.2">
+      <c r="A2" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="70.8">
+      <c r="A3" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>398</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="72">
+      <c r="A4" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" t="s">
+        <v>401</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="57.6">
+      <c r="A5" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" t="s">
+        <v>399</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="86.4">
+      <c r="A6" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" t="s">
+        <v>402</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="72">
+      <c r="A7" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J7" t="s">
+        <v>400</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="99.6">
+      <c r="A8" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J8" t="s">
+        <v>403</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="86.4">
+      <c r="A9" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>371</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>371</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J9" t="s">
+        <v>404</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="86.4">
+      <c r="A10" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J10" t="s">
+        <v>405</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="86.4">
+      <c r="A11" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J11" t="s">
+        <v>406</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="86.4">
+      <c r="A12" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J12" t="s">
+        <v>407</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="86.4">
+      <c r="A13" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J13" t="s">
+        <v>408</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>396</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C5A01BE-886C-4DDC-81AD-947C5C4E69CA}">
   <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -5135,7 +6707,7 @@
       </c>
     </row>
     <row r="4" spans="1:12" ht="187.2">
-      <c r="B4" s="15">
+      <c r="B4" s="14">
         <v>46283</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -5175,12 +6747,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E116B88-DD8B-45A5-9B4A-BCF42512281C}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" customWidth="1"/>
+    <col min="1" max="1" width="25.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="28.8">
@@ -5201,25 +6773,72 @@
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="4"/>
+      <c r="A2" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="B2" s="2">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="4"/>
+      <c r="A3" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="B3" s="2">
+        <v>13</v>
+      </c>
+      <c r="C3" s="2">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="4"/>
+      <c r="A4" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="B4" s="2">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2">
+        <v>6</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>324</v>
+      </c>
+      <c r="B5" s="2">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2">
+        <v>12</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: add persistent metadata append mechanism
* Add firmware metadata update states
* Add persistent metadata record structure with sequence tracking
* Add CRC validation using STM32 hardware CRC peripheral
* Add commit marker for incomplete-write detection
* Implement latest valid metadata record lookup
* Implement append-only metadata record programming
* Preserve previous valid metadata records during state updates
* Support independent metadata histories for Slot A and Slot B
* Detect and ignore incomplete or corrupted metadata records

This establishes the metadata persistence foundation for the FOTA update-state and recovery flow.
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A320F884-4DEF-48E9-97F6-3D4986577E91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69DABBE8-D7F1-4CB5-B3BD-DA19CD5794C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project_Info" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,9 @@
     <sheet name="Memory_Linked_Config_Test" sheetId="9" r:id="rId3"/>
     <sheet name="Dual_Image_FOTA_Test" sheetId="10" r:id="rId4"/>
     <sheet name="FOTA Boot Flow Validation" sheetId="11" r:id="rId5"/>
-    <sheet name="Defect_Log" sheetId="4" r:id="rId6"/>
-    <sheet name="Test_Summary" sheetId="5" r:id="rId7"/>
+    <sheet name="FOTA_Metadata_Append" sheetId="12" r:id="rId6"/>
+    <sheet name="Defect_Log" sheetId="4" r:id="rId7"/>
+    <sheet name="Test_Summary" sheetId="5" r:id="rId8"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="481">
   <si>
     <t>Field</t>
   </si>
@@ -4605,6 +4606,360 @@
   </si>
   <si>
     <t>FOTA-VAL-012_Active_SHA256_Mismatch.png</t>
+  </si>
+  <si>
+    <t>FOTA-META-001</t>
+  </si>
+  <si>
+    <t>Metadata Record Creation</t>
+  </si>
+  <si>
+    <t>System shall create a valid persistent metadata record</t>
+  </si>
+  <si>
+    <t>Verify that the first metadata record can be appended to an erased metadata sector</t>
+  </si>
+  <si>
+    <t>Slot A metadata sector is erased; valid firmware metadata is available</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Write a metadata record with sequence = 1 and state = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CONFIRMED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; read the sector back</t>
+    </r>
+  </si>
+  <si>
+    <t>Record is programmed successfully; sequence = 1; metadata fields match; CRC is valid; commit marker is valid</t>
+  </si>
+  <si>
+    <t>FOTA-META-001_First_Record.png</t>
+  </si>
+  <si>
+    <t>Initial append test</t>
+  </si>
+  <si>
+    <t>FOTA-META-002</t>
+  </si>
+  <si>
+    <t>Metadata Record Readback</t>
+  </si>
+  <si>
+    <t>System shall identify the latest valid metadata record</t>
+  </si>
+  <si>
+    <t>Verify that the first committed record can be read correctly</t>
+  </si>
+  <si>
+    <t>FOTA-META-001 passed</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Execute </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Metadata_ReadLatestRecord()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> on Slot A metadata sector</t>
+    </r>
+  </si>
+  <si>
+    <t>Function returns the sequence-1 record and correct firmware metadata</t>
+  </si>
+  <si>
+    <t>FOTA-META-002_Read_First_Record.png</t>
+  </si>
+  <si>
+    <t>Verify read path</t>
+  </si>
+  <si>
+    <t>FOTA-META-003</t>
+  </si>
+  <si>
+    <t>Metadata State Append</t>
+  </si>
+  <si>
+    <t>System shall append a new metadata state without modifying the previous record</t>
+  </si>
+  <si>
+    <t>Verify that a second state is appended instead of overwriting Record 0</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Record 0 exists with state </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CONFIRMED</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Create identical metadata with state </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>BOOT_PENDING</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; call </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Metadata_WriteRecord()</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Record 1 is created with sequence = 2; Record 0 remains unchanged; latest record reports </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>BOOT_PENDING</t>
+    </r>
+  </si>
+  <si>
+    <t>FOTA-META-003_State_Append.png</t>
+  </si>
+  <si>
+    <t>Confirms append-only behavior</t>
+  </si>
+  <si>
+    <t>FOTA-META-004</t>
+  </si>
+  <si>
+    <t>Metadata CRC Validation</t>
+  </si>
+  <si>
+    <t>System shall detect corrupted metadata records</t>
+  </si>
+  <si>
+    <t>Verify CRC detects modification of a committed record</t>
+  </si>
+  <si>
+    <t>A valid committed metadata record exists</t>
+  </si>
+  <si>
+    <t>Modify one metadata field in the stored record using debugger/GDB; read and validate the record</t>
+  </si>
+  <si>
+    <r>
+      <t>Metadata_ValidateRecord()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> rejects the modified record because calculated CRC differs from stored CRC</t>
+    </r>
+  </si>
+  <si>
+    <t>FOTA-META-004_CRC_Mismatch.png</t>
+  </si>
+  <si>
+    <t>Tests corruption detection</t>
+  </si>
+  <si>
+    <t>FOTA-META-005</t>
+  </si>
+  <si>
+    <t>Commit Marker Validation</t>
+  </si>
+  <si>
+    <t>System shall reject an incomplete metadata record</t>
+  </si>
+  <si>
+    <t>Verify that a record without a valid commit marker is ignored</t>
+  </si>
+  <si>
+    <t>Record 0 and Record 1 are valid; next record location is erased</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Create/program a metadata record but leave </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>commit_marker = 0xFFFFFFFFU</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; run </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Metadata_ReadLatestRecord()</t>
+    </r>
+  </si>
+  <si>
+    <t>Incomplete record is ignored; previous valid record remains the latest record</t>
+  </si>
+  <si>
+    <t>FOTA-META-005_Commit_Marker_Invalid.png</t>
+  </si>
+  <si>
+    <t>Simulates interrupted metadata write</t>
+  </si>
+  <si>
+    <t>FOTA-META-006</t>
+  </si>
+  <si>
+    <t>Sequence Handling</t>
+  </si>
+  <si>
+    <t>System shall select the newest valid metadata record</t>
+  </si>
+  <si>
+    <t>Verify sequence number determines the latest state</t>
+  </si>
+  <si>
+    <t>Multiple valid records exist in the metadata sector</t>
+  </si>
+  <si>
+    <t>Read the metadata sector containing sequence 1 and sequence 2 valid records</t>
+  </si>
+  <si>
+    <t>Sequence 2 is returned as the latest valid record</t>
+  </si>
+  <si>
+    <t>FOTA-META-006_Sequence_Selection.png</t>
+  </si>
+  <si>
+    <t>Confirms journal ordering</t>
+  </si>
+  <si>
+    <t>FOTA-META-007</t>
+  </si>
+  <si>
+    <t>Slot B Metadata Append</t>
+  </si>
+  <si>
+    <t>Slot A and Slot B shall maintain independent metadata histories</t>
+  </si>
+  <si>
+    <t>Verify the append mechanism works independently for Slot B</t>
+  </si>
+  <si>
+    <t>Slot B metadata sector is erased; valid Slot B firmware metadata is available</t>
+  </si>
+  <si>
+    <t>Write an initial Slot B record and then append a second state</t>
+  </si>
+  <si>
+    <t>Slot B records are stored and read independently without affecting Slot A metadata</t>
+  </si>
+  <si>
+    <t>FOTA-META-007_Slot_B_Append.png</t>
+  </si>
+  <si>
+    <t>Confirms A/B metadata separation</t>
+  </si>
+  <si>
+    <t>FOTA-META-008</t>
+  </si>
+  <si>
+    <t>Multiple Append Operations</t>
+  </si>
+  <si>
+    <t>Metadata state changes shall be stored as sequential records</t>
+  </si>
+  <si>
+    <t>Verify repeated state changes can be appended without erasing the sector</t>
+  </si>
+  <si>
+    <t>Metadata sector has sufficient erased records</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Append several valid states sequentially, for example </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>PENDING_VALIDATION → VALIDATED → BOOT_PENDING</t>
+    </r>
+  </si>
+  <si>
+    <t>Each state is stored as a new record with an incremented sequence; latest valid state is returned</t>
+  </si>
+  <si>
+    <t>FOTA-META-008_Multiple_Appends.png</t>
+  </si>
+  <si>
+    <t>Establishes journal behavior before FOTA integration</t>
   </si>
 </sst>
 </file>
@@ -6573,6 +6928,312 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D653C8DE-C68F-48B6-8D4E-947E06745D0D}">
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="8.5546875" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" customWidth="1"/>
+    <col min="3" max="3" width="19" customWidth="1"/>
+    <col min="4" max="4" width="22.44140625" customWidth="1"/>
+    <col min="5" max="5" width="20.21875" customWidth="1"/>
+    <col min="6" max="6" width="31.44140625" customWidth="1"/>
+    <col min="7" max="7" width="28.44140625" customWidth="1"/>
+    <col min="8" max="8" width="20.5546875" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" customWidth="1"/>
+    <col min="10" max="10" width="15.44140625" customWidth="1"/>
+    <col min="11" max="11" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="43.2">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="57.6">
+      <c r="A2" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="43.2">
+      <c r="A3" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="57.6">
+      <c r="A4" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="57.6">
+      <c r="A5" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>442</v>
+      </c>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="6" t="s">
+        <v>443</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="57.6">
+      <c r="A6" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="6" t="s">
+        <v>452</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="43.2">
+      <c r="A7" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="57.6">
+      <c r="A8" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="57.6">
+      <c r="A9" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="6" t="s">
+        <v>479</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>480</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C5A01BE-886C-4DDC-81AD-947C5C4E69CA}">
   <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
@@ -6747,7 +7408,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E116B88-DD8B-45A5-9B4A-BCF42512281C}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.4"/>

</xml_diff>

<commit_message>
feat: add A/B firmware confirmation and metadata tooling
- Implement firmware confirmation for Slot A and Slot B
- Add watchdog protection for trial firmware
- Remove obsolete candidate-based flash programming APIs
- Add host-side Python metadata generation tool
- Add STM32-compatible metadata CRC generation
- Document metadata programming and GDB workflow
- Record current flash programming/debugging procedure and observed issues
- Preserve current fail-safe issue for investigation before validation
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69DABBE8-D7F1-4CB5-B3BD-DA19CD5794C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87EAE5D3-5B69-437E-BF46-F9D0B271B213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project_Info" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="587">
   <si>
     <t>Field</t>
   </si>
@@ -4960,6 +4960,940 @@
   </si>
   <si>
     <t>Establishes journal behavior before FOTA integration</t>
+  </si>
+  <si>
+    <t>DIF-007</t>
+  </si>
+  <si>
+    <t>Slot A Normal Boot</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Bootloader shall boot Slot A when Slot A metadata is valid, Slot A image is valid, and Slot A is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CONFIRMED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Verify normal boot of the confirmed Slot A firmware in the new A/B architecture.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Valid Slot A image at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08020000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; valid Slot A metadata in Sector 2; latest Slot A state = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CONFIRMED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; Slot B may be empty.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Flash valid Slot A image. 2. Program valid Slot A metadata. 3. Reset MCU. 4. Observe bootloader decision. 5. Verify SCB-&gt;VTOR and PC using GDB. 6. Verify Slot A application executes.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Bootloader selects Slot A; metadata and SHA-256 validation succeed; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>JumpToApplication()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> executes; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>SCB-&gt;VTOR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08020000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; PC lies within Slot A region; Slot A executes normally.</t>
+    </r>
+  </si>
+  <si>
+    <t>DIF-007_Slot_A_Normal_Boot.png</t>
+  </si>
+  <si>
+    <t>First baseline test for the finalized A/B architecture.</t>
+  </si>
+  <si>
+    <t>DIF-008</t>
+  </si>
+  <si>
+    <t>Slot B Normal Boot</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Bootloader shall boot Slot B when Slot B metadata is valid, Slot B image is valid, and Slot B is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CONFIRMED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Verify normal boot of the confirmed Slot B firmware.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Valid Slot B image at </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08040000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; valid Slot B metadata in Sector 3; latest Slot B state = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CONFIRMED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; Slot A may be empty.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Flash valid Slot B image. 2. Program valid Slot B metadata. 3. Reset MCU. 4. Observe bootloader decision. 5. Verify SCB-&gt;VTOR and PC. 6. Verify Slot B application executes.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Bootloader selects Slot B; integrity verification succeeds; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>SCB-&gt;VTOR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>0x08040000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; PC lies within Slot B region; Slot B executes normally.</t>
+    </r>
+  </si>
+  <si>
+    <t>DIF-008_Slot_B_Normal_Boot.png</t>
+  </si>
+  <si>
+    <t>Verifies the second physical firmware slot.</t>
+  </si>
+  <si>
+    <t>DIF-009</t>
+  </si>
+  <si>
+    <t>Active Slot Selection</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Bootloader shall select the slot whose latest valid metadata state is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CONFIRMED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Verify that active-slot selection is state-driven rather than version-driven.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Slot A latest record = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CONFIRMED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; Slot B latest record = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>EMPTY</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> or no valid record.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Reset MCU. 2. Inspect Slot A and Slot B metadata records. 3. Observe active-slot selection. 4. Verify selected image and PC.</t>
+  </si>
+  <si>
+    <t>Slot A is selected as active regardless of version comparison; Slot B is treated as inactive.</t>
+  </si>
+  <si>
+    <t>DIF-009_Active_Slot_Selection_A.png</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Confirms </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CONFIRMED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> state is the boot-selection criterion.</t>
+    </r>
+  </si>
+  <si>
+    <t>DIF-010</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Bootloader shall select Slot B when Slot B is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CONFIRMED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and Slot A is not active.</t>
+    </r>
+  </si>
+  <si>
+    <t>Verify reverse A/B active-slot selection.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Slot B latest record = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CONFIRMED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; Slot A latest record = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ROLLBACK</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>INVALID</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>EMPTY</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, or no valid record.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Reset MCU. 2. Inspect both metadata states. 3. Observe selected slot. 4. Verify Slot B execution.</t>
+  </si>
+  <si>
+    <t>Slot B is selected as active and Slot A is treated as inactive.</t>
+  </si>
+  <si>
+    <t>DIF-010_Active_Slot_Selection_B.png</t>
+  </si>
+  <si>
+    <t>Confirms the architecture works in both directions.</t>
+  </si>
+  <si>
+    <t>DIF-011</t>
+  </si>
+  <si>
+    <t>Inactive Slot Isolation</t>
+  </si>
+  <si>
+    <t>Invalid inactive-slot metadata shall not prevent the confirmed active slot from booting.</t>
+  </si>
+  <si>
+    <t>Verify that only the selected confirmed slot is required for normal boot integrity validation.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Slot A = valid </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CONFIRMED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; Slot B metadata intentionally corrupted.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Corrupt Slot B metadata. 2. Reset MCU. 3. Observe bootloader metadata handling. 4. Verify Slot A integrity check. 5. Verify Slot A execution.</t>
+  </si>
+  <si>
+    <t>Bootloader identifies Slot A as confirmed; invalid Slot B metadata does not block Slot A validation or execution.</t>
+  </si>
+  <si>
+    <t>DIF-011_Invalid_Inactive_Metadata.png</t>
+  </si>
+  <si>
+    <t>Important distinction from the earlier active/candidate architecture.</t>
+  </si>
+  <si>
+    <t>DIF-012</t>
+  </si>
+  <si>
+    <t>Metadata Record Validation</t>
+  </si>
+  <si>
+    <t>Bootloader/application shall accept a metadata record only when commit marker and CRC are valid.</t>
+  </si>
+  <si>
+    <t>Verify persistent metadata record integrity.</t>
+  </si>
+  <si>
+    <t>Valid metadata record exists in Slot A or Slot B metadata sector.</t>
+  </si>
+  <si>
+    <t>1. Read latest metadata record. 2. Verify commit marker. 3. Recalculate CRC. 4. Compare against stored CRC.</t>
+  </si>
+  <si>
+    <t>Valid record is accepted as a valid metadata record.</t>
+  </si>
+  <si>
+    <t>DIF-012_Metadata_Record_Validation.png</t>
+  </si>
+  <si>
+    <t>Uses the new append-record format.</t>
+  </si>
+  <si>
+    <t>DIF-013</t>
+  </si>
+  <si>
+    <t>Metadata CRC Corruption</t>
+  </si>
+  <si>
+    <t>System shall reject a metadata record when its stored CRC does not match the calculated CRC.</t>
+  </si>
+  <si>
+    <t>Verify detection of metadata corruption.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Valid metadata record exists; stored </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>metadata_crc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is modified.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Corrupt </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>metadata_crc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> using GDB. 2. Reset MCU. 3. Read metadata sector. 4. Observe record validation.</t>
+    </r>
+  </si>
+  <si>
+    <t>Corrupted record is rejected and not selected as the latest valid record.</t>
+  </si>
+  <si>
+    <t>DIF-013_Metadata_CRC_Corruption.png</t>
+  </si>
+  <si>
+    <t>First direct negative test of the new CRC mechanism.</t>
+  </si>
+  <si>
+    <t>DIF-014</t>
+  </si>
+  <si>
+    <t>System shall reject an incomplete metadata record when the commit marker is invalid or erased.</t>
+  </si>
+  <si>
+    <t>Verify incomplete-record protection.</t>
+  </si>
+  <si>
+    <t>Valid record exists or a test record is partially programmed.</t>
+  </si>
+  <si>
+    <t>1. Remove/corrupt the commit marker. 2. Reset MCU. 3. Scan metadata records.</t>
+  </si>
+  <si>
+    <t>Record without the correct commit marker is ignored as invalid.</t>
+  </si>
+  <si>
+    <t>DIF-014_Metadata_Commit_Marker_Corruption.png</t>
+  </si>
+  <si>
+    <t>Demonstrates commit marker being the final record-validity condition.</t>
+  </si>
+  <si>
+    <t>DIF-015</t>
+  </si>
+  <si>
+    <t>Metadata Sequence Handling</t>
+  </si>
+  <si>
+    <t>System shall select the newest valid metadata record based on sequence number.</t>
+  </si>
+  <si>
+    <t>Verify append-journal selection logic.</t>
+  </si>
+  <si>
+    <t>Multiple valid records exist in a metadata sector with different sequence numbers.</t>
+  </si>
+  <si>
+    <t>1. Create multiple valid records with increasing sequence numbers. 2. Reset MCU. 3. Read latest record. 4. Inspect returned sequence/state.</t>
+  </si>
+  <si>
+    <t>Highest valid sequence is selected as the latest metadata record.</t>
+  </si>
+  <si>
+    <t>DIF-015_Metadata_Sequence_Handling.png</t>
+  </si>
+  <si>
+    <t>Confirms historical records remain intact while latest state is selected.</t>
+  </si>
+  <si>
+    <t>DIF-016</t>
+  </si>
+  <si>
+    <t>Slot Confirmation</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Slot firmware shall change </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>BOOT_PENDING</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CONFIRMED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> after successful startup confirmation.</t>
+    </r>
+  </si>
+  <si>
+    <t>Verify application-side trial firmware confirmation.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Slot A image is valid and its latest metadata state is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>BOOT_PENDING</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; Slot B remains the previous confirmed/inactive state as applicable.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Start Slot A with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>BOOT_PENDING</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. 2. Allow startup to execute </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Firmware_Confirm()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. 3. Read Slot A metadata sector. 4. Inspect latest sequence and state.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">New metadata record is appended; latest state becomes </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CONFIRMED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; previous </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>BOOT_PENDING</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> record remains unchanged.</t>
+    </r>
+  </si>
+  <si>
+    <t>DIF-016_Slot_A_Firmware_Confirmation.png</t>
+  </si>
+  <si>
+    <t>Verifies application-side confirmation using the common metadata journal.</t>
+  </si>
+  <si>
+    <t>DIF-017</t>
+  </si>
+  <si>
+    <t>Watchdog Protection</t>
+  </si>
+  <si>
+    <t>Trial firmware shall not continuously refresh the watchdog before successful confirmation.</t>
+  </si>
+  <si>
+    <t>Verify watchdog protects an unconfirmed trial firmware.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Slot A is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>BOOT_PENDING</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; IWDG enabled; confirmation path intentionally prevented.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Start Slot A trial firmware. 2. Prevent successful confirmation. 3. Do not service IWDG after the configured timeout. 4. Observe MCU reset.</t>
+  </si>
+  <si>
+    <t>IWDG expires and automatically resets the MCU.</t>
+  </si>
+  <si>
+    <t>DIF-017_Watchdog_Trial_Reset.png</t>
+  </si>
+  <si>
+    <t>Core failed-trial test; bootloader fallback is tested separately.</t>
+  </si>
+  <si>
+    <t>DIF-018</t>
+  </si>
+  <si>
+    <t>Watchdog Normal Operation</t>
+  </si>
+  <si>
+    <t>Confirmed firmware shall service the watchdog during normal operation.</t>
+  </si>
+  <si>
+    <t>Verify watchdog does not cause unintended resets during healthy operation.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Slot A latest state = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CONFIRMED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; IWDG enabled.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Boot Slot A normally. 2. Allow application to run for a sustained period. 3. Monitor reset behavior.</t>
+  </si>
+  <si>
+    <t>Watchdog is refreshed within the timeout and no watchdog reset occurs during healthy operation.</t>
+  </si>
+  <si>
+    <t>DIF-018_Watchdog_Normal_Operation.png</t>
+  </si>
+  <si>
+    <t>Establishes the normal watchdog baseline before failure testing.</t>
   </si>
 </sst>
 </file>
@@ -6182,7 +7116,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD30C987-18E6-4B70-93B6-FCBA274DBA4D}">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="13"/>
@@ -6441,6 +7375,378 @@
       </c>
       <c r="K7" s="2" t="s">
         <v>301</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="115.2">
+      <c r="A8" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="6" t="s">
+        <v>488</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="86.4">
+      <c r="A9" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="6" t="s">
+        <v>497</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="72">
+      <c r="A10" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="86.4">
+      <c r="A11" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="6" t="s">
+        <v>514</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="86.4">
+      <c r="A12" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="6" t="s">
+        <v>523</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="86.4">
+      <c r="A13" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="86.4">
+      <c r="A14" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="6" t="s">
+        <v>541</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="100.8">
+      <c r="A15" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="6" t="s">
+        <v>549</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="72">
+      <c r="A16" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>557</v>
+      </c>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="6" t="s">
+        <v>558</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="100.8">
+      <c r="A17" s="2" t="s">
+        <v>560</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="6" t="s">
+        <v>567</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="100.8">
+      <c r="A18" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="72">
+      <c r="A19" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>580</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="6" t="s">
+        <v>585</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>586</v>
       </c>
     </row>
   </sheetData>
@@ -6945,7 +8251,7 @@
     <col min="11" max="11" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="43.2">
+    <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
@@ -7104,7 +8410,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="57.6">
+    <row r="6" spans="1:11" ht="56.4">
       <c r="A6" s="2" t="s">
         <v>445</v>
       </c>
@@ -7230,6 +8536,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
test: complete A/B FOTA validation and recovery testing
Completed functional validation of the dual-slot A/B FOTA update and recovery workflow.

- Verified consecutive A → B → A → B firmware update cycling.
- Validated firmware metadata, image boundaries, SHA-256 integrity, and candidate confirmation.
- Tested interrupted destination programming and recovery through automatic update retry.
- Verified rollback to the previously confirmed firmware when a candidate fails to confirm or triggers a watchdog reset.
- Validated confirmed image persistence and reuse of a previously failed slot for subsequent updates.
- Verified BootSafe entry when the active firmware fails SHA-256 integrity verification.
- Executed the defined FOTA test cases and collected supporting test evidence.
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC892F78-BB95-452C-98EC-E8EC44B6DB44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64FBEA09-C762-4A77-A6F8-9AA41C8E205A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,21 +18,31 @@
     <sheet name="Memory_Linked_Config_Test" sheetId="9" r:id="rId3"/>
     <sheet name="Dual_Image_FOTA_Test" sheetId="10" r:id="rId4"/>
     <sheet name="FOTA Boot Flow Validation" sheetId="11" r:id="rId5"/>
-    <sheet name="FOTA_Metadata_Append" sheetId="12" r:id="rId6"/>
+    <sheet name="FOTA_AB_Cycling_Recovery" sheetId="13" r:id="rId6"/>
     <sheet name="Defect_Log" sheetId="4" r:id="rId7"/>
     <sheet name="Test_Summary" sheetId="5" r:id="rId8"/>
+    <sheet name="COMMON_GDB_ERROR" sheetId="14" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="768" uniqueCount="615">
   <si>
     <t>Field</t>
   </si>
@@ -4494,358 +4504,7 @@
     <t>FOTA-VAL-012_Active_SHA256_Mismatch.png</t>
   </si>
   <si>
-    <t>FOTA-META-001</t>
-  </si>
-  <si>
-    <t>Metadata Record Creation</t>
-  </si>
-  <si>
-    <t>System shall create a valid persistent metadata record</t>
-  </si>
-  <si>
-    <t>Verify that the first metadata record can be appended to an erased metadata sector</t>
-  </si>
-  <si>
-    <t>Slot A metadata sector is erased; valid firmware metadata is available</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Write a metadata record with sequence = 1 and state = </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>CONFIRMED</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>; read the sector back</t>
-    </r>
-  </si>
-  <si>
-    <t>Record is programmed successfully; sequence = 1; metadata fields match; CRC is valid; commit marker is valid</t>
-  </si>
-  <si>
-    <t>FOTA-META-001_First_Record.png</t>
-  </si>
-  <si>
-    <t>Initial append test</t>
-  </si>
-  <si>
-    <t>FOTA-META-002</t>
-  </si>
-  <si>
-    <t>Metadata Record Readback</t>
-  </si>
-  <si>
-    <t>System shall identify the latest valid metadata record</t>
-  </si>
-  <si>
-    <t>Verify that the first committed record can be read correctly</t>
-  </si>
-  <si>
-    <t>FOTA-META-001 passed</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Execute </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Metadata_ReadLatestRecord()</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> on Slot A metadata sector</t>
-    </r>
-  </si>
-  <si>
-    <t>Function returns the sequence-1 record and correct firmware metadata</t>
-  </si>
-  <si>
-    <t>FOTA-META-002_Read_First_Record.png</t>
-  </si>
-  <si>
-    <t>Verify read path</t>
-  </si>
-  <si>
-    <t>FOTA-META-003</t>
-  </si>
-  <si>
-    <t>Metadata State Append</t>
-  </si>
-  <si>
-    <t>System shall append a new metadata state without modifying the previous record</t>
-  </si>
-  <si>
-    <t>Verify that a second state is appended instead of overwriting Record 0</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Record 0 exists with state </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>CONFIRMED</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Create identical metadata with state </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>BOOT_PENDING</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">; call </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Metadata_WriteRecord()</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Record 1 is created with sequence = 2; Record 0 remains unchanged; latest record reports </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>BOOT_PENDING</t>
-    </r>
-  </si>
-  <si>
-    <t>FOTA-META-003_State_Append.png</t>
-  </si>
-  <si>
-    <t>Confirms append-only behavior</t>
-  </si>
-  <si>
-    <t>FOTA-META-004</t>
-  </si>
-  <si>
-    <t>Metadata CRC Validation</t>
-  </si>
-  <si>
-    <t>System shall detect corrupted metadata records</t>
-  </si>
-  <si>
-    <t>Verify CRC detects modification of a committed record</t>
-  </si>
-  <si>
-    <t>A valid committed metadata record exists</t>
-  </si>
-  <si>
-    <t>Modify one metadata field in the stored record using debugger/GDB; read and validate the record</t>
-  </si>
-  <si>
-    <r>
-      <t>Metadata_ValidateRecord()</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> rejects the modified record because calculated CRC differs from stored CRC</t>
-    </r>
-  </si>
-  <si>
-    <t>FOTA-META-004_CRC_Mismatch.png</t>
-  </si>
-  <si>
-    <t>Tests corruption detection</t>
-  </si>
-  <si>
-    <t>FOTA-META-005</t>
-  </si>
-  <si>
     <t>Commit Marker Validation</t>
-  </si>
-  <si>
-    <t>System shall reject an incomplete metadata record</t>
-  </si>
-  <si>
-    <t>Verify that a record without a valid commit marker is ignored</t>
-  </si>
-  <si>
-    <t>Record 0 and Record 1 are valid; next record location is erased</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Create/program a metadata record but leave </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>commit_marker = 0xFFFFFFFFU</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">; run </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>Metadata_ReadLatestRecord()</t>
-    </r>
-  </si>
-  <si>
-    <t>Incomplete record is ignored; previous valid record remains the latest record</t>
-  </si>
-  <si>
-    <t>FOTA-META-005_Commit_Marker_Invalid.png</t>
-  </si>
-  <si>
-    <t>Simulates interrupted metadata write</t>
-  </si>
-  <si>
-    <t>FOTA-META-006</t>
-  </si>
-  <si>
-    <t>Sequence Handling</t>
-  </si>
-  <si>
-    <t>System shall select the newest valid metadata record</t>
-  </si>
-  <si>
-    <t>Verify sequence number determines the latest state</t>
-  </si>
-  <si>
-    <t>Multiple valid records exist in the metadata sector</t>
-  </si>
-  <si>
-    <t>Read the metadata sector containing sequence 1 and sequence 2 valid records</t>
-  </si>
-  <si>
-    <t>Sequence 2 is returned as the latest valid record</t>
-  </si>
-  <si>
-    <t>FOTA-META-006_Sequence_Selection.png</t>
-  </si>
-  <si>
-    <t>Confirms journal ordering</t>
-  </si>
-  <si>
-    <t>FOTA-META-007</t>
-  </si>
-  <si>
-    <t>Slot B Metadata Append</t>
-  </si>
-  <si>
-    <t>Slot A and Slot B shall maintain independent metadata histories</t>
-  </si>
-  <si>
-    <t>Verify the append mechanism works independently for Slot B</t>
-  </si>
-  <si>
-    <t>Slot B metadata sector is erased; valid Slot B firmware metadata is available</t>
-  </si>
-  <si>
-    <t>Write an initial Slot B record and then append a second state</t>
-  </si>
-  <si>
-    <t>Slot B records are stored and read independently without affecting Slot A metadata</t>
-  </si>
-  <si>
-    <t>FOTA-META-007_Slot_B_Append.png</t>
-  </si>
-  <si>
-    <t>Confirms A/B metadata separation</t>
-  </si>
-  <si>
-    <t>FOTA-META-008</t>
-  </si>
-  <si>
-    <t>Multiple Append Operations</t>
-  </si>
-  <si>
-    <t>Metadata state changes shall be stored as sequential records</t>
-  </si>
-  <si>
-    <t>Verify repeated state changes can be appended without erasing the sector</t>
-  </si>
-  <si>
-    <t>Metadata sector has sufficient erased records</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Append several valid states sequentially, for example </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>PENDING_VALIDATION → VALIDATED → BOOT_PENDING</t>
-    </r>
-  </si>
-  <si>
-    <t>Each state is stored as a new record with an incremented sequence; latest valid state is returned</t>
-  </si>
-  <si>
-    <t>FOTA-META-008_Multiple_Appends.png</t>
-  </si>
-  <si>
-    <t>Establishes journal behavior before FOTA integration</t>
   </si>
   <si>
     <t>DIF-007</t>
@@ -5324,12 +4983,1125 @@
   <si>
     <t xml:space="preserve">Secure Boot - Firmware Integrity Verification </t>
   </si>
+  <si>
+    <t>A/B Update Cycling</t>
+  </si>
+  <si>
+    <t>FOTA-AB-001</t>
+  </si>
+  <si>
+    <t>A → B Update</t>
+  </si>
+  <si>
+    <t>FOTA-AB-002</t>
+  </si>
+  <si>
+    <t>B → A Update</t>
+  </si>
+  <si>
+    <t>FOTA-AB-003</t>
+  </si>
+  <si>
+    <t>FOTA-AB-004</t>
+  </si>
+  <si>
+    <t>Full A → B → A → B Cycling</t>
+  </si>
+  <si>
+    <t>FOTA-AB-005</t>
+  </si>
+  <si>
+    <t>Interrupted Programming</t>
+  </si>
+  <si>
+    <t>FOTA-AB-006</t>
+  </si>
+  <si>
+    <t>Interrupted Update</t>
+  </si>
+  <si>
+    <t>FOTA-AB-007</t>
+  </si>
+  <si>
+    <t>Interrupted Metadata/Commit Programming</t>
+  </si>
+  <si>
+    <t>FOTA-AB-008</t>
+  </si>
+  <si>
+    <t>Failed Confirmation</t>
+  </si>
+  <si>
+    <t>FOTA-AB-009</t>
+  </si>
+  <si>
+    <t>Watchdog Reset During Candidate Boot</t>
+  </si>
+  <si>
+    <t>FOTA-AB-010</t>
+  </si>
+  <si>
+    <t>Repeated Watchdog Recovery</t>
+  </si>
+  <si>
+    <t>FOTA-AB-011</t>
+  </si>
+  <si>
+    <t>Confirmed Image Persistence</t>
+  </si>
+  <si>
+    <t>FOTA-AB-012</t>
+  </si>
+  <si>
+    <t>Recovery Followed by New Update</t>
+  </si>
+  <si>
+    <t>FOTA-AB-013</t>
+  </si>
+  <si>
+    <t>FOTA-AB-014</t>
+  </si>
+  <si>
+    <t>Active Slot Recovery</t>
+  </si>
+  <si>
+    <t>FOTA-AB-015</t>
+  </si>
+  <si>
+    <t>FOTA-AB-016</t>
+  </si>
+  <si>
+    <t>The bootloader shall boot a valid confirmed active firmware image before an A/B update cycle is initiated.</t>
+  </si>
+  <si>
+    <t>Establish a known-good baseline before executing A/B cycling tests.</t>
+  </si>
+  <si>
+    <t>Power-cycle or reset the device and observe the bootloader decision and running firmware identifier.</t>
+  </si>
+  <si>
+    <t>Baseline for subsequent tests.</t>
+  </si>
+  <si>
+    <t>The bootloader shall support updating the device from a valid confirmed Slot A image to a valid candidate image in Slot B.</t>
+  </si>
+  <si>
+    <t>Verify a successful update from Slot A to Slot B.</t>
+  </si>
+  <si>
+    <r>
+      <t>FW-A1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is active and confirmed; valid </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is available in the download/staging area.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Program </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; generate/program its metadata; reset the device; allow candidate validation and boot; complete firmware confirmation.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>FW-B1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> passes validation, boots from Slot B, and becomes the confirmed active firmware.</t>
+    </r>
+  </si>
+  <si>
+    <t>Uses existing candidate validation and confirmation mechanisms.</t>
+  </si>
+  <si>
+    <t>The bootloader shall support updating the device from a valid confirmed Slot B image to a valid candidate image in Slot A.</t>
+  </si>
+  <si>
+    <t>Verify a successful return update from Slot B to Slot A.</t>
+  </si>
+  <si>
+    <r>
+      <t>FW-B1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is active and confirmed; valid </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-A2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is available in the download/staging area.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Program </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-A2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; generate/program metadata; reset; validate and boot Slot A; complete confirmation.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>FW-A2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> boots successfully from Slot A and becomes the confirmed active firmware.</t>
+    </r>
+  </si>
+  <si>
+    <t>Verifies reverse-direction slot reuse.</t>
+  </si>
+  <si>
+    <t>The bootloader shall allow a previously used Slot B to accept a subsequent valid firmware update after Slot A has become active.</t>
+  </si>
+  <si>
+    <t>Verify reuse of Slot B for a second update.</t>
+  </si>
+  <si>
+    <r>
+      <t>FW-A2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is active and confirmed; valid </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is available.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Program </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; perform validation; reset; boot Slot B; complete confirmation.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>FW-B2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> boots successfully from Slot B and becomes the confirmed active firmware.</t>
+    </r>
+  </si>
+  <si>
+    <t>Confirms repeated reuse of Slot B.</t>
+  </si>
+  <si>
+    <t>The FOTA mechanism shall support consecutive successful firmware updates between Slot A and Slot B without reprogramming the bootloader.</t>
+  </si>
+  <si>
+    <t>Validate complete A/B cycling across multiple consecutive updates.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Valid </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-A1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-A2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> images are available.</t>
+    </r>
+  </si>
+  <si>
+    <t>Execute the A→B, B→A, and A→B update sequences sequentially.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The device successfully completes </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>A1 → B1 → A2 → B2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; the correct slot is selected after each reset; final active firmware is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Primary end-to-end A/B cycling test.</t>
+  </si>
+  <si>
+    <t>The FOTA mechanism shall recover safely when programming of a candidate image is interrupted before the image is completely written.</t>
+  </si>
+  <si>
+    <t>Verify recovery from an incomplete candidate firmware programming operation.</t>
+  </si>
+  <si>
+    <r>
+      <t>FW-A1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is active and confirmed; Slot B is the update target.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Start programming </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; interrupt programming using reset or power removal before completion; restore power.</t>
+    </r>
+  </si>
+  <si>
+    <t>The incomplete Slot B image is rejected and the last confirmed Slot A firmware remains bootable and active.</t>
+  </si>
+  <si>
+    <t>Perform interruption during image programming.</t>
+  </si>
+  <si>
+    <t>The FOTA mechanism shall not activate a candidate image when an update is interrupted before activation is completed.</t>
+  </si>
+  <si>
+    <t>Verify recovery when the image is completely written but activation/commit is interrupted.</t>
+  </si>
+  <si>
+    <r>
+      <t>FW-A1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is active and confirmed; complete </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is available.</t>
+    </r>
+  </si>
+  <si>
+    <t>Program the complete candidate image; interrupt/reset the device before activation or commit is finalized.</t>
+  </si>
+  <si>
+    <t>The uncommitted Slot B image is not selected as the active image; the previously confirmed Slot A image boots.</t>
+  </si>
+  <si>
+    <t>Validates transactional update behavior.</t>
+  </si>
+  <si>
+    <t>The FOTA mechanism shall recover from an interruption during candidate metadata or commit-marker programming.</t>
+  </si>
+  <si>
+    <t>Verify that partially programmed update metadata cannot cause an invalid boot decision.</t>
+  </si>
+  <si>
+    <r>
+      <t>FW-A1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is active and confirmed; valid </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is being installed.</t>
+    </r>
+  </si>
+  <si>
+    <t>Interrupt power/reset during metadata, state-record, or commit-marker programming.</t>
+  </si>
+  <si>
+    <t>Incomplete or invalid metadata is rejected and the last valid confirmed Slot A firmware is selected.</t>
+  </si>
+  <si>
+    <t>Reference metadata append, CRC, and commit validation tests.</t>
+  </si>
+  <si>
+    <t>The FOTA mechanism shall revert to the previously confirmed firmware when a newly booted candidate image fails to confirm.</t>
+  </si>
+  <si>
+    <t>Verify rollback after candidate confirmation failure.</t>
+  </si>
+  <si>
+    <r>
+      <t>FW-A1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is confirmed; valid </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is selected for candidate boot.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Boot </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; prevent the application from issuing the required confirmation; reset the device.</t>
+    </r>
+  </si>
+  <si>
+    <t>Slot B is treated as unconfirmed/failed and the previously confirmed Slot A image is restored as the boot target.</t>
+  </si>
+  <si>
+    <t>Candidate may execute temporarily but must not remain permanently active.</t>
+  </si>
+  <si>
+    <t>The FOTA mechanism shall recover when a candidate firmware image causes a watchdog reset before successful confirmation.</t>
+  </si>
+  <si>
+    <t>Verify recovery from watchdog-triggered candidate failure.</t>
+  </si>
+  <si>
+    <r>
+      <t>FW-A1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is confirmed; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is selected as candidate; watchdog mechanism is enabled.</t>
+    </r>
+  </si>
+  <si>
+    <t>Execute a test candidate that intentionally stops servicing the watchdog; allow the watchdog to reset the device.</t>
+  </si>
+  <si>
+    <t>After reset, the bootloader detects unsuccessful candidate execution/confirmation and boots the previously confirmed Slot A image.</t>
+  </si>
+  <si>
+    <t>Evidence should include watchdog reset and subsequent Slot A boot.</t>
+  </si>
+  <si>
+    <t>The FOTA mechanism shall prevent an unsuccessful candidate image from causing an indefinite reboot loop.</t>
+  </si>
+  <si>
+    <t>Verify recovery after repeated candidate watchdog failures.</t>
+  </si>
+  <si>
+    <r>
+      <t>FW-A1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is confirmed; failing </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is available for candidate boot.</t>
+    </r>
+  </si>
+  <si>
+    <t>Allow the failing candidate to boot and watchdog-reset repeatedly according to the configured recovery mechanism.</t>
+  </si>
+  <si>
+    <t>The bootloader eventually abandons the failing candidate and boots the last confirmed Slot A image; no infinite candidate reboot loop occurs.</t>
+  </si>
+  <si>
+    <t>Applicable when retry/attempt handling is implemented.</t>
+  </si>
+  <si>
+    <t>A successfully confirmed firmware image shall remain the active boot image across subsequent resets and power cycles until another valid update is accepted.</t>
+  </si>
+  <si>
+    <t>Verify persistence of a successfully confirmed Slot B image.</t>
+  </si>
+  <si>
+    <r>
+      <t>FW-B1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> has been successfully confirmed as active.</t>
+    </r>
+  </si>
+  <si>
+    <t>Perform multiple software resets and power cycles without initiating another update.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Slot B remains selected and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> boots successfully after every reset and power cycle.</t>
+    </r>
+  </si>
+  <si>
+    <t>Demonstrates persistence of successful activation.</t>
+  </si>
+  <si>
+    <t>After recovering from a failed candidate update, the FOTA mechanism shall allow the previously failed slot to be reused for a subsequent valid firmware update.</t>
+  </si>
+  <si>
+    <t>Verify that recovery does not leave the failed slot unusable.</t>
+  </si>
+  <si>
+    <t>Slot A is confirmed after recovery; Slot B contains a previously failed candidate.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Recover to Slot A; replace the failed Slot B image with valid </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-B2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; perform a new update and confirmation.</t>
+    </r>
+  </si>
+  <si>
+    <t>Slot A boots successfully after recovery, and the new valid Slot B image is subsequently accepted and confirmed.</t>
+  </si>
+  <si>
+    <t>Important recovery-to-normal-operation test.</t>
+  </si>
+  <si>
+    <t>Reverse-direction interruption test.</t>
+  </si>
+  <si>
+    <t>Deliberately corrupt firmware contents in Slot B; reset the device.</t>
+  </si>
+  <si>
+    <t>References existing active SHA-256 verification tests.</t>
+  </si>
+  <si>
+    <t>Demonstrates continued FOTA operation after fault recovery.</t>
+  </si>
+  <si>
+    <t>FOTA-AB-002_SlotA_to_SlotB_SuccessfulUpdate.png</t>
+  </si>
+  <si>
+    <t>FOTA-AB-003_SlotB_to_SlotA_SuccessfulUpdate.png</t>
+  </si>
+  <si>
+    <t>FOTA-AB-004_SlotA_to_SlotB_SecondUpdate.png</t>
+  </si>
+  <si>
+    <t>FOTA-AB-005_A_to_B_to_A_to_B_Cycle.png</t>
+  </si>
+  <si>
+    <t>FOTA-AB-006_InterruptedProgramming_Recovery.png</t>
+  </si>
+  <si>
+    <t>FOTA-AB-007_InterruptedActivation_Recovery.png</t>
+  </si>
+  <si>
+    <t>FOTA-AB-008_InterruptedMetadataCommit_Recovery.png</t>
+  </si>
+  <si>
+    <t>FOTA-AB-009_CandidateConfirmationFailure_Rollback.png</t>
+  </si>
+  <si>
+    <t>FOTA-AB-010_WatchdogReset_CandidateRecovery.png</t>
+  </si>
+  <si>
+    <t>FOTA-AB-011_RepeatedWatchdog_NoBootLoop.png</t>
+  </si>
+  <si>
+    <t>FOTA-AB-012_ConfirmedImage_Persistence.png</t>
+  </si>
+  <si>
+    <t>FOTA-AB-013_Recovery_then_NewUpdate.png</t>
+  </si>
+  <si>
+    <t>FOTA-AB-014_InterruptedB_to_A_Recovery.png</t>
+  </si>
+  <si>
+    <t>FOTA-AB-015_ActiveSlotIntegrityFailure_Fallback.png</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Bootloader is programmed; Slot A contains valid confirmed </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-A1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; device is operational.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Slot A is selected and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FW-A1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> executes successfully.</t>
+    </r>
+  </si>
+  <si>
+    <t>FOTA-AB-001_ActiveSlotA_ConfirmedBoot.png</t>
+  </si>
+  <si>
+    <t>call FlashStorage_ProgramImage(0x08010000, 0x20010000, 15024)</t>
+  </si>
+  <si>
+    <t>$10 = HAL_BUSY</t>
+  </si>
+  <si>
+    <t>Error</t>
+  </si>
+  <si>
+    <t>Diagnosis</t>
+  </si>
+  <si>
+    <t>p pFlash.Lock</t>
+  </si>
+  <si>
+    <t>$11 = HAL_LOCKED</t>
+  </si>
+  <si>
+    <t>p pFlash.ProcedureOnGoing</t>
+  </si>
+  <si>
+    <t>$12 = FLASH_PROC_NONE</t>
+  </si>
+  <si>
+    <t>x/wx 0x40023C0C</t>
+  </si>
+  <si>
+    <t>0x40023c0c: 0x00000000</t>
+  </si>
+  <si>
+    <t>x/wx 0x40023C10</t>
+  </si>
+  <si>
+    <t>0x40023c10: 0x80000000</t>
+  </si>
+  <si>
+    <t>set var pFlash.Lock = 0</t>
+  </si>
+  <si>
+    <t>$13 = HAL_UNLOCKED</t>
+  </si>
+  <si>
+    <t>$14 = HAL_OK</t>
+  </si>
+  <si>
+    <t>x/8wx 0x08010000</t>
+  </si>
+  <si>
+    <t>0x8010000: 0x20020000 0x08040e81 0x08040cb1 0x08040cb9</t>
+  </si>
+  <si>
+    <t>0x8010010: 0x08040cc1 0x08040cc9 0x08040cd1 0x00000000</t>
+  </si>
+  <si>
+    <t>The HAL's internal software lock is held</t>
+  </si>
+  <si>
+    <t>No flash procedure is marked as ongoing</t>
+  </si>
+  <si>
+    <t>No busy or error flags are set in the status register</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The flash controller's </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>LOCK</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> bit is set</t>
+    </r>
+  </si>
+  <si>
+    <t>Interrupted A → B Update and Recovery</t>
+  </si>
+  <si>
+    <t>The FOTA mechanism shall preserve the last confirmed Slot A image and recover safely when programming an update targeting Slot B is interrupted.</t>
+  </si>
+  <si>
+    <t>Verify preservation of the confirmed firmware and recovery through automatic update retry after interrupted destination programming.</t>
+  </si>
+  <si>
+    <t>FW-A1 is active and confirmed in Slot A. A valid FW-B2 image is available in the staging area with valid metadata and SHA-256.</t>
+  </si>
+  <si>
+    <t>Start programming FW-B2 into Slot B. Interrupt destination programming using a debugger reset before programming completes. Allow the bootloader to restart and process the pending update.before completion; reset/power-cycle the device.</t>
+  </si>
+  <si>
+    <t>Slot A remains intact, and its firmware integrity verification succeeds. The bootloader revalidates the staged image and retries programming Slot B. If the retry succeeds, the destination SHA-256 matches, Slot B boots as a candidate, and firmware confirmation completes successfully.</t>
+  </si>
+  <si>
+    <t>Slot B integrity verification fails and the bootloader selects and boots BootSafe firmware.</t>
+  </si>
+  <si>
+    <t>Slot B is active and confirmed.</t>
+  </si>
+  <si>
+    <t>Verify active-slot recovery using the BootSafe Mechanism.</t>
+  </si>
+  <si>
+    <t>The bootloader shall fall back to BootSafe mode when the currently active firmware fails integrity verification.</t>
+  </si>
+  <si>
+    <t>Active Slot Selection After Reset</t>
+  </si>
+  <si>
+    <t>After reset, the bootloader shall select the previously configured active firmware slot and perform integrity verification before execution.</t>
+  </si>
+  <si>
+    <t>Verify that the bootloader consistently selects the configured active slot after reset.</t>
+  </si>
+  <si>
+    <t>Slot B is configured as the active slot. Slot A contains a valid firmware image.</t>
+  </si>
+  <si>
+    <t>Reset the device and observe the bootloader's active-slot selection and integrity verification.</t>
+  </si>
+  <si>
+    <t>The bootloader selects Slot B and verifies its SHA-256. If Slot B remains corrupted, the integrity check fails and the bootloader enters fail-safe mode, as specified by the current implementation.</t>
+  </si>
+  <si>
+    <t>FOTA-AB-016_ActiveSlotSelection_AfterReset.png</t>
+  </si>
+  <si>
+    <t>FOTA_AB_Cycling_Recovery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5358,6 +6130,18 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF00FF00"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -5379,7 +6163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -5389,9 +6173,6 @@
     </xf>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -5420,8 +6201,23 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5724,7 +6520,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>518</v>
+        <v>447</v>
       </c>
     </row>
     <row r="4" spans="2:3">
@@ -6011,12 +6807,12 @@
       <c r="B9" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6039,7 +6835,7 @@
     <col min="6" max="6" width="23.77734375" customWidth="1"/>
     <col min="7" max="7" width="22.109375" customWidth="1"/>
     <col min="8" max="8" width="22.44140625" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" style="11"/>
+    <col min="9" max="9" width="8.88671875" style="10"/>
     <col min="10" max="10" width="23.88671875" customWidth="1"/>
     <col min="11" max="11" width="17.33203125" customWidth="1"/>
   </cols>
@@ -6104,10 +6900,10 @@
       <c r="H2" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="5" t="s">
         <v>94</v>
       </c>
       <c r="K2" s="2" t="s">
@@ -6136,13 +6932,13 @@
       <c r="G3" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="I3" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="5" t="s">
         <v>104</v>
       </c>
       <c r="K3" s="2" t="s">
@@ -6171,13 +6967,13 @@
       <c r="G4" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="I4" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="5" t="s">
         <v>112</v>
       </c>
       <c r="K4" s="2" t="s">
@@ -6206,13 +7002,13 @@
       <c r="G5" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="I5" s="10" t="s">
+      <c r="I5" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="5" t="s">
         <v>123</v>
       </c>
       <c r="K5" s="2" t="s">
@@ -6244,10 +7040,10 @@
       <c r="H6" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="I6" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="J6" s="5" t="s">
         <v>132</v>
       </c>
       <c r="K6" s="2" t="s">
@@ -6279,10 +7075,10 @@
       <c r="H7" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="I7" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J7" s="6" t="s">
+      <c r="J7" s="5" t="s">
         <v>162</v>
       </c>
       <c r="K7" s="2" t="s">
@@ -6314,10 +7110,10 @@
       <c r="H8" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J8" s="6" t="s">
+      <c r="J8" s="5" t="s">
         <v>172</v>
       </c>
       <c r="K8" s="2" t="s">
@@ -6346,13 +7142,13 @@
       <c r="G9" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="I9" s="10" t="s">
+      <c r="I9" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="J9" s="5" t="s">
         <v>182</v>
       </c>
       <c r="K9" s="2" t="s">
@@ -6381,156 +7177,156 @@
       <c r="G10" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="H10" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="I10" s="10" t="s">
+      <c r="I10" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J10" s="6" t="s">
+      <c r="J10" s="5" t="s">
         <v>192</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="11" spans="1:11" s="8" customFormat="1" ht="115.2">
-      <c r="A11" s="8" t="s">
+    <row r="11" spans="1:11" s="7" customFormat="1" ht="115.2">
+      <c r="A11" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="8" t="s">
         <v>205</v>
       </c>
-      <c r="I11" s="10" t="s">
+      <c r="I11" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="J11" s="8" t="s">
         <v>204</v>
       </c>
-      <c r="K11" s="7" t="s">
+      <c r="K11" s="6" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="12" spans="1:11" s="7" customFormat="1" ht="129.6">
-      <c r="A12" s="7" t="s">
+    <row r="12" spans="1:11" s="6" customFormat="1" ht="129.6">
+      <c r="A12" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="I12" s="10" t="s">
+      <c r="I12" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J12" s="7" t="s">
+      <c r="J12" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="K12" s="7" t="s">
+      <c r="K12" s="6" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="13" spans="1:11" s="7" customFormat="1" ht="144">
-      <c r="A13" s="7" t="s">
+    <row r="13" spans="1:11" s="6" customFormat="1" ht="144">
+      <c r="A13" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="6" t="s">
         <v>220</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="G13" s="7" t="s">
+      <c r="G13" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="I13" s="10" t="s">
+      <c r="I13" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J13" s="7" t="s">
+      <c r="J13" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="K13" s="7" t="s">
+      <c r="K13" s="6" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="14" spans="1:11" s="7" customFormat="1" ht="100.8">
-      <c r="A14" s="7" t="s">
+    <row r="14" spans="1:11" s="6" customFormat="1" ht="100.8">
+      <c r="A14" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="I14" s="10" t="s">
+      <c r="I14" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J14" s="7" t="s">
+      <c r="J14" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="K14" s="7" t="s">
+      <c r="K14" s="6" t="s">
         <v>222</v>
       </c>
     </row>
@@ -6545,7 +7341,7 @@
   <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="12"/>
+    <col min="1" max="1" width="8.88671875" style="11"/>
     <col min="2" max="2" width="10.5546875" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="22.77734375" customWidth="1"/>
@@ -6553,7 +7349,7 @@
     <col min="6" max="6" width="41.21875" customWidth="1"/>
     <col min="7" max="7" width="22.6640625" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" style="11"/>
+    <col min="9" max="9" width="8.88671875" style="10"/>
     <col min="10" max="10" width="16.21875" customWidth="1"/>
     <col min="11" max="11" width="17.6640625" customWidth="1"/>
   </cols>
@@ -6594,7 +7390,7 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="115.2">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>233</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -6612,13 +7408,13 @@
       <c r="F2" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="9" t="s">
         <v>33</v>
       </c>
       <c r="J2" s="2" t="s">
@@ -6680,7 +7476,7 @@
         <v>254</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>512</v>
+        <v>441</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>255</v>
@@ -6715,7 +7511,7 @@
         <v>266</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>508</v>
+        <v>437</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>267</v>
@@ -6726,7 +7522,7 @@
       <c r="I5" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="5" t="s">
         <v>269</v>
       </c>
       <c r="K5" s="2" t="s">
@@ -6750,7 +7546,7 @@
         <v>283</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>509</v>
+        <v>438</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>284</v>
@@ -6761,7 +7557,7 @@
       <c r="I6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="J6" s="5" t="s">
         <v>287</v>
       </c>
       <c r="K6" s="2" t="s">
@@ -6785,7 +7581,7 @@
         <v>292</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>507</v>
+        <v>436</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>293</v>
@@ -6805,107 +7601,107 @@
     </row>
     <row r="8" spans="1:11" ht="115.2">
       <c r="A8" s="2" t="s">
-        <v>475</v>
+        <v>404</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>476</v>
+        <v>405</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>477</v>
+        <v>406</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>478</v>
+        <v>407</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>479</v>
+        <v>408</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>506</v>
+        <v>435</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>480</v>
+        <v>409</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>505</v>
+        <v>434</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="J8" s="6" t="s">
-        <v>481</v>
+      <c r="J8" s="5" t="s">
+        <v>410</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>482</v>
+        <v>411</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="100.8">
       <c r="A9" s="2" t="s">
-        <v>483</v>
+        <v>412</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>485</v>
+        <v>414</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>486</v>
+        <v>415</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>487</v>
+        <v>416</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>488</v>
+        <v>417</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>510</v>
+        <v>439</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>489</v>
+        <v>418</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>489</v>
+        <v>418</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="J9" s="6" t="s">
-        <v>513</v>
+      <c r="J9" s="5" t="s">
+        <v>442</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>490</v>
+        <v>419</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="100.8">
       <c r="A10" s="2" t="s">
-        <v>484</v>
+        <v>413</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>440</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>491</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>492</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>493</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>511</v>
-      </c>
       <c r="G10" s="2" t="s">
-        <v>494</v>
+        <v>423</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>494</v>
+        <v>423</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="6" t="s">
-        <v>514</v>
+      <c r="J10" s="5" t="s">
+        <v>443</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>495</v>
+        <v>424</v>
       </c>
     </row>
   </sheetData>
@@ -6985,10 +7781,10 @@
       <c r="F2" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="5" t="s">
         <v>323</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="5" t="s">
         <v>323</v>
       </c>
       <c r="I2" s="2" t="s">
@@ -7020,16 +7816,16 @@
       <c r="F3" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>329</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="4" t="s">
         <v>392</v>
       </c>
       <c r="K3" s="2" t="s">
@@ -7055,10 +7851,10 @@
       <c r="F4" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="5" t="s">
         <v>335</v>
       </c>
       <c r="I4" s="2" t="s">
@@ -7090,10 +7886,10 @@
       <c r="F5" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="5" t="s">
         <v>341</v>
       </c>
       <c r="I5" s="2" t="s">
@@ -7125,10 +7921,10 @@
       <c r="F6" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="5" t="s">
         <v>348</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="5" t="s">
         <v>348</v>
       </c>
       <c r="I6" s="2" t="s">
@@ -7230,10 +8026,10 @@
       <c r="F9" s="2" t="s">
         <v>364</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="5" t="s">
         <v>365</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="5" t="s">
         <v>365</v>
       </c>
       <c r="I9" s="2" t="s">
@@ -7393,21 +8189,19 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D653C8DE-C68F-48B6-8D4E-947E06745D0D}">
-  <dimension ref="A1:K9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CC24105-2E09-406B-BCFD-ABDBD3411BFF}">
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="8.5546875" customWidth="1"/>
-    <col min="2" max="2" width="10.6640625" customWidth="1"/>
-    <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="22.44140625" customWidth="1"/>
-    <col min="5" max="5" width="20.21875" customWidth="1"/>
-    <col min="6" max="6" width="31.44140625" customWidth="1"/>
-    <col min="7" max="7" width="28.44140625" customWidth="1"/>
-    <col min="8" max="8" width="20.5546875" customWidth="1"/>
-    <col min="9" max="9" width="9.33203125" customWidth="1"/>
-    <col min="10" max="10" width="15.44140625" customWidth="1"/>
-    <col min="11" max="11" width="15.21875" customWidth="1"/>
+    <col min="2" max="2" width="10.77734375" customWidth="1"/>
+    <col min="3" max="3" width="26.33203125" customWidth="1"/>
+    <col min="4" max="4" width="23" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="22.88671875" customWidth="1"/>
+    <col min="7" max="7" width="21.88671875" customWidth="1"/>
+    <col min="8" max="8" width="24.21875" customWidth="1"/>
+    <col min="10" max="10" width="18.6640625" customWidth="1"/>
+    <col min="11" max="11" width="15.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -7445,257 +8239,568 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="57.6">
+    <row r="2" spans="1:11" ht="72">
       <c r="A2" s="2" t="s">
-        <v>403</v>
+        <v>449</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>404</v>
+        <v>448</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>405</v>
+        <v>477</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>406</v>
+        <v>478</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>407</v>
+        <v>571</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>408</v>
+        <v>479</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>409</v>
-      </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="6" t="s">
-        <v>410</v>
+        <v>572</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>573</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="43.2">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="100.8">
       <c r="A3" s="2" t="s">
-        <v>412</v>
+        <v>451</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>413</v>
+        <v>450</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>414</v>
+        <v>481</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>416</v>
+        <v>482</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>483</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>417</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>418</v>
-      </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="6" t="s">
-        <v>419</v>
+        <v>484</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>557</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="57.6">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="72">
       <c r="A4" s="2" t="s">
-        <v>421</v>
+        <v>453</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>422</v>
+        <v>452</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>423</v>
+        <v>487</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>424</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>425</v>
+        <v>488</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>489</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>426</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>427</v>
-      </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="6" t="s">
-        <v>428</v>
+        <v>490</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>558</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="57.6">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="72">
       <c r="A5" s="2" t="s">
-        <v>430</v>
+        <v>454</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>431</v>
+        <v>450</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>432</v>
+        <v>493</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>434</v>
+        <v>494</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>495</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>436</v>
-      </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="6" t="s">
-        <v>437</v>
+        <v>496</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>559</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="56.4">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="86.4">
       <c r="A6" s="2" t="s">
-        <v>439</v>
+        <v>456</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>440</v>
+        <v>455</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>441</v>
+        <v>499</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>442</v>
+        <v>500</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>443</v>
+        <v>501</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>444</v>
+        <v>502</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>445</v>
-      </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="6" t="s">
-        <v>446</v>
+        <v>503</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>560</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="43.2">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="86.4">
       <c r="A7" s="2" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>449</v>
+        <v>457</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>450</v>
+        <v>505</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>451</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>452</v>
+        <v>506</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>507</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>453</v>
+        <v>508</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>454</v>
-      </c>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="6" t="s">
-        <v>455</v>
+        <v>509</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>561</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="57.6">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="72">
       <c r="A8" s="2" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>459</v>
+        <v>511</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>460</v>
-      </c>
-      <c r="E8" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="72">
+      <c r="A9" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>462</v>
-      </c>
-      <c r="G8" s="2" t="s">
+      <c r="C9" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>563</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="86.4">
+      <c r="A10" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="6" t="s">
-        <v>464</v>
-      </c>
-      <c r="K8" s="2" t="s">
+      <c r="C10" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>525</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>564</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="86.4">
+      <c r="A11" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>465</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" ht="57.6">
-      <c r="A9" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="B9" s="2" t="s">
+      <c r="C11" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>531</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>565</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="100.8">
+      <c r="A12" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="C12" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>537</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>566</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="86.4">
+      <c r="A13" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>469</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="F9" s="2" t="s">
+      <c r="C13" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>543</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>567</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="86.4">
+      <c r="A14" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>471</v>
       </c>
-      <c r="G9" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="6" t="s">
+      <c r="C14" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>568</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="187.2">
+      <c r="A15" s="2" t="s">
         <v>473</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="B15" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>598</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>599</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>600</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>569</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="72">
+      <c r="A16" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>474</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>570</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="129.6">
+      <c r="A17" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>606</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>607</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>612</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>556</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7704,19 +8809,19 @@
   <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" style="5" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.33203125" style="5" customWidth="1"/>
-    <col min="4" max="4" width="21" style="5" customWidth="1"/>
-    <col min="5" max="5" width="27" style="5" customWidth="1"/>
-    <col min="6" max="6" width="17.21875" style="5" customWidth="1"/>
-    <col min="7" max="7" width="29.5546875" style="5" customWidth="1"/>
-    <col min="8" max="8" width="20.21875" style="5" customWidth="1"/>
-    <col min="9" max="9" width="14" style="5" customWidth="1"/>
-    <col min="10" max="10" width="19.44140625" style="5" customWidth="1"/>
-    <col min="11" max="11" width="7.5546875" style="5" customWidth="1"/>
-    <col min="12" max="12" width="14.77734375" style="5" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="1" width="12.5546875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="21" style="4" customWidth="1"/>
+    <col min="5" max="5" width="27" style="4" customWidth="1"/>
+    <col min="6" max="6" width="17.21875" style="4" customWidth="1"/>
+    <col min="7" max="7" width="29.5546875" style="4" customWidth="1"/>
+    <col min="8" max="8" width="20.21875" style="4" customWidth="1"/>
+    <col min="9" max="9" width="14" style="4" customWidth="1"/>
+    <col min="10" max="10" width="19.44140625" style="4" customWidth="1"/>
+    <col min="11" max="11" width="7.5546875" style="4" customWidth="1"/>
+    <col min="12" max="12" width="14.77734375" style="4" customWidth="1"/>
+    <col min="13" max="16384" width="8.88671875" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="28.8">
@@ -7761,7 +8866,7 @@
       <c r="A2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="12">
         <v>46276</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -7799,7 +8904,7 @@
       <c r="A3" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="12">
         <v>46280</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -7817,7 +8922,7 @@
       <c r="G3" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>148</v>
       </c>
       <c r="I3" s="2" t="s">
@@ -7834,10 +8939,10 @@
       </c>
     </row>
     <row r="4" spans="1:12" ht="187.2">
-      <c r="A4" s="11" t="s">
-        <v>502</v>
-      </c>
-      <c r="B4" s="13">
+      <c r="A4" s="10" t="s">
+        <v>431</v>
+      </c>
+      <c r="B4" s="12">
         <v>46283</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -7847,7 +8952,7 @@
         <v>273</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>503</v>
+        <v>432</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>274</v>
@@ -7871,42 +8976,42 @@
         <v>279</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="230.4">
-      <c r="A5" s="11" t="s">
-        <v>501</v>
-      </c>
-      <c r="B5" s="13">
+    <row r="5" spans="1:12" ht="216">
+      <c r="A5" s="10" t="s">
+        <v>430</v>
+      </c>
+      <c r="B5" s="12">
         <v>46298</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>496</v>
+        <v>425</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>497</v>
+        <v>426</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>504</v>
+        <v>433</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>498</v>
+        <v>427</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>499</v>
+        <v>428</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>515</v>
+        <v>444</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>500</v>
+        <v>429</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>516</v>
+        <v>445</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>70</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>517</v>
+        <v>446</v>
       </c>
     </row>
   </sheetData>
@@ -7917,10 +9022,11 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E116B88-DD8B-45A5-9B4A-BCF42512281C}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="25.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="5" width="8.88671875" style="10"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="28.8">
@@ -7944,16 +9050,16 @@
       <c r="A2" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="9">
         <v>5</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="9">
         <v>5</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="9">
         <v>0</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="17">
         <v>1</v>
       </c>
     </row>
@@ -7961,16 +9067,16 @@
       <c r="A3" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="9">
         <v>13</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="9">
         <v>13</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="9">
         <v>0</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="17">
         <v>1</v>
       </c>
     </row>
@@ -7978,16 +9084,16 @@
       <c r="A4" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="9">
         <v>6</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="9">
         <v>6</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="9">
         <v>0</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="17">
         <v>1</v>
       </c>
     </row>
@@ -7995,20 +9101,181 @@
       <c r="A5" t="s">
         <v>318</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="9">
         <v>12</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="9">
         <v>12</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="9">
         <v>0</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>613</v>
+      </c>
+      <c r="B6" s="9">
+        <v>16</v>
+      </c>
+      <c r="C6" s="9">
+        <v>16</v>
+      </c>
+      <c r="D6" s="9">
+        <v>0</v>
+      </c>
+      <c r="E6" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="16" t="s">
+        <v>614</v>
+      </c>
+      <c r="B7" s="10">
+        <f>B2+B3+B4+B5+B6</f>
+        <v>52</v>
+      </c>
+      <c r="C7" s="10">
+        <f>SUM(C2:C6)</f>
+        <v>52</v>
+      </c>
+      <c r="D7" s="9">
+        <v>0</v>
+      </c>
+      <c r="E7" s="18">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7CFF7B5-6090-47FE-9CE6-89A61875E880}">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="2" max="2" width="64.109375" customWidth="1"/>
+    <col min="3" max="3" width="64" customWidth="1"/>
+    <col min="4" max="4" width="49.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="B1" t="s">
+        <v>576</v>
+      </c>
+      <c r="C1" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>574</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="B3" s="14" t="s">
+        <v>575</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>579</v>
+      </c>
+      <c r="D3" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="C4" s="13" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="C5" s="14" t="s">
+        <v>581</v>
+      </c>
+      <c r="D5" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="C6" s="13" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="C7" s="14" t="s">
+        <v>583</v>
+      </c>
+      <c r="D7" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="C8" s="13" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="C9" s="14" t="s">
+        <v>585</v>
+      </c>
+      <c r="D9" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="C10" s="13" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="C11" s="13" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="C12" s="14" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="C13" s="13" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="C14" s="14" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="C15" s="13" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="C16" s="14" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3">
+      <c r="C17" s="14" t="s">
+        <v>591</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>